<commit_message>
Cập nhật file OM4-DE-IS-0010.xlsx qua web
</commit_message>
<xml_diff>
--- a/du-lieu/OM4-DE-IS-0010.xlsx
+++ b/du-lieu/OM4-DE-IS-0010.xlsx
@@ -13,9 +13,9 @@
     <workbookView xWindow="-11520" yWindow="-21720" windowWidth="51840" windowHeight="21120" tabRatio="667" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Detailed PL" sheetId="5" r:id="rId1"/>
-    <sheet name="Commercial Invoice" sheetId="1" r:id="rId2"/>
-    <sheet name="Break Down CI" sheetId="2" r:id="rId3"/>
+    <sheet name="Break Down CI" sheetId="2" r:id="rId1"/>
+    <sheet name="Detailed PL" sheetId="5" r:id="rId2"/>
+    <sheet name="Commercial Invoice" sheetId="1" r:id="rId3"/>
     <sheet name="Packing List (1_2)" sheetId="3" r:id="rId4"/>
     <sheet name="PL(2_2)" sheetId="4" r:id="rId5"/>
     <sheet name="SHIPPING MARK (001)" sheetId="12" r:id="rId6"/>
@@ -35,170 +35,170 @@
     <externalReference r:id="rId18"/>
   </externalReferences>
   <definedNames>
+    <definedName name="__123Graph_A" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_A" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_A" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="__123Graph_A" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_A" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_A" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_A" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_A" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_A" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="__123Graph_ACurrent" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_ACurrent" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_ACurrent" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="__123Graph_ACurrent" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_ACurrent" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_ACurrent" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_ACurrent" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_ACurrent" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_ACurrent" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="__123Graph_B" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_B" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_B" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="__123Graph_B" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_B" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_B" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_B" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_B" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_B" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="__123Graph_BCurrent" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_BCurrent" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_BCurrent" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="__123Graph_BCurrent" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_BCurrent" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_BCurrent" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_BCurrent" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_BCurrent" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_BCurrent" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="__123Graph_D" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_D" localSheetId="2" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_D" localSheetId="1" hidden="1">#REF!</definedName>
-    <definedName name="__123Graph_D" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_D" localSheetId="3" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_D" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_D" localSheetId="6" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_D" hidden="1">#REF!</definedName>
+    <definedName name="__123Graph_E" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_E" localSheetId="2" hidden="1">#REF!</definedName>
-    <definedName name="__123Graph_E" localSheetId="1" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_E" localSheetId="3" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_E" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_E" localSheetId="6" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_E" hidden="1">#REF!</definedName>
+    <definedName name="__123Graph_LBL_A" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_LBL_A" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_LBL_A" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="__123Graph_LBL_A" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_LBL_A" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_LBL_A" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_LBL_A" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_LBL_A" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_LBL_A" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="__123Graph_LBL_B" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_LBL_B" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_LBL_B" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="__123Graph_LBL_B" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_LBL_B" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_LBL_B" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_LBL_B" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_LBL_B" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_LBL_B" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="__123Graph_X" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_X" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_X" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="__123Graph_X" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_X" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_X" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_X" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_X" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_X" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="__123Graph_XCurrent" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_XCurrent" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_XCurrent" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="__123Graph_XCurrent" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_XCurrent" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_XCurrent" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_XCurrent" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="__123Graph_XCurrent" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="__123Graph_XCurrent" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="_1__123Graph_AChart_1A" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_1__123Graph_AChart_1A" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_1__123Graph_AChart_1A" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="_1__123Graph_AChart_1A" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_1__123Graph_AChart_1A" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_1__123Graph_AChart_1A" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_1__123Graph_AChart_1A" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_1__123Graph_AChart_1A" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="_1__123Graph_AChart_1A" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="_2__123Graph_BChart_1A" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_2__123Graph_BChart_1A" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_2__123Graph_BChart_1A" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="_2__123Graph_BChart_1A" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_2__123Graph_BChart_1A" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_2__123Graph_BChart_1A" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_2__123Graph_BChart_1A" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_2__123Graph_BChart_1A" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="_2__123Graph_BChart_1A" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="_3__123Graph_XChart_1A" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_3__123Graph_XChart_1A" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_3__123Graph_XChart_1A" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="_3__123Graph_XChart_1A" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_3__123Graph_XChart_1A" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_3__123Graph_XChart_1A" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_3__123Graph_XChart_1A" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="_3__123Graph_XChart_1A" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="_3__123Graph_XChart_1A" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="_Fill" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="_Fill" localSheetId="2" hidden="1">#REF!</definedName>
     <definedName name="_Fill" localSheetId="1" hidden="1">#REF!</definedName>
-    <definedName name="_Fill" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="_Fill" localSheetId="3" hidden="1">#REF!</definedName>
     <definedName name="_Fill" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="_Fill" localSheetId="6" hidden="1">#REF!</definedName>
     <definedName name="_Fill" hidden="1">#REF!</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Break Down CI'!$A$8:$N$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Detailed PL'!$B$13:$AH$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Break Down CI'!$A$8:$P$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed PL'!$B$13:$AH$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'SHIPPING MARK (001)'!$A$1:$A$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'SHIPPING MARK (2)'!$A$1:$A$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Technical Description'!$A$8:$H$11</definedName>
     <definedName name="_Hlk215568700" localSheetId="11">PSIC!$B$2</definedName>
+    <definedName name="_Key1" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="_Key1" localSheetId="2" hidden="1">#REF!</definedName>
-    <definedName name="_Key1" localSheetId="1" hidden="1">#REF!</definedName>
     <definedName name="_Key1" localSheetId="3" hidden="1">#REF!</definedName>
     <definedName name="_Key1" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="_Key1" localSheetId="6" hidden="1">#REF!</definedName>
     <definedName name="_Key1" hidden="1">#REF!</definedName>
+    <definedName name="_Key2" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="_Key2" localSheetId="2" hidden="1">#REF!</definedName>
-    <definedName name="_Key2" localSheetId="1" hidden="1">#REF!</definedName>
     <definedName name="_Key2" localSheetId="3" hidden="1">#REF!</definedName>
     <definedName name="_Key2" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="_Key2" localSheetId="6" hidden="1">#REF!</definedName>
     <definedName name="_Key2" hidden="1">#REF!</definedName>
     <definedName name="_Order1" hidden="1">255</definedName>
     <definedName name="_Order2" hidden="1">255</definedName>
+    <definedName name="_Parse_In" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="_Parse_In" localSheetId="2" hidden="1">#REF!</definedName>
     <definedName name="_Parse_In" localSheetId="1" hidden="1">#REF!</definedName>
-    <definedName name="_Parse_In" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="_Parse_In" localSheetId="3" hidden="1">#REF!</definedName>
     <definedName name="_Parse_In" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="_Parse_In" localSheetId="6" hidden="1">#REF!</definedName>
     <definedName name="_Parse_In" hidden="1">#REF!</definedName>
+    <definedName name="_Parse_Out" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="_Parse_Out" localSheetId="2" hidden="1">#REF!</definedName>
-    <definedName name="_Parse_Out" localSheetId="1" hidden="1">#REF!</definedName>
     <definedName name="_Parse_Out" localSheetId="3" hidden="1">#REF!</definedName>
     <definedName name="_Parse_Out" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="_Parse_Out" localSheetId="6" hidden="1">#REF!</definedName>
     <definedName name="_Parse_Out" hidden="1">#REF!</definedName>
+    <definedName name="_Sort" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="_Sort" localSheetId="2" hidden="1">#REF!</definedName>
-    <definedName name="_Sort" localSheetId="1" hidden="1">#REF!</definedName>
     <definedName name="_Sort" localSheetId="3" hidden="1">#REF!</definedName>
     <definedName name="_Sort" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="_Sort" localSheetId="6" hidden="1">#REF!</definedName>
     <definedName name="_Sort" hidden="1">#REF!</definedName>
+    <definedName name="A" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="A" localSheetId="2" hidden="1">#REF!</definedName>
-    <definedName name="A" localSheetId="1" hidden="1">#REF!</definedName>
     <definedName name="A" localSheetId="3" hidden="1">#REF!</definedName>
     <definedName name="A" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="A" localSheetId="6" hidden="1">#REF!</definedName>
     <definedName name="A" hidden="1">#REF!</definedName>
+    <definedName name="ABC" localSheetId="0" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ABC" localSheetId="2" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ABC" localSheetId="1" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="ABC" localSheetId="0" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ABC" localSheetId="3" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ABC" localSheetId="5" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ABC" localSheetId="6" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ABC" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="ABC" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="CO" localSheetId="0" hidden="1">'[3]Eq. Mobilization'!#REF!</definedName>
     <definedName name="CO" localSheetId="2" hidden="1">'[3]Eq. Mobilization'!#REF!</definedName>
     <definedName name="CO" localSheetId="1" hidden="1">'[3]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="CO" localSheetId="0" hidden="1">'[3]Eq. Mobilization'!#REF!</definedName>
     <definedName name="CO" localSheetId="3" hidden="1">'[3]Eq. Mobilization'!#REF!</definedName>
     <definedName name="CO" localSheetId="5" hidden="1">'[3]Eq. Mobilization'!#REF!</definedName>
     <definedName name="CO" localSheetId="6" hidden="1">'[3]Eq. Mobilization'!#REF!</definedName>
@@ -212,25 +212,25 @@
     <definedName name="Ge" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="Ge" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="Ge" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="iv2dt" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="iv2dt" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="iv2dt" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="iv2dt" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="iv2dt" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="iv2dt" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="iv2dt" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="iv2dt" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="iv2dt" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="ivdt" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ivdt" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ivdt" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="ivdt" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ivdt" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ivdt" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ivdt" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ivdt" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="ivdt" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="KABOLINE" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="KABOLINE" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="KABOLINE" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="KABOLINE" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="KABOLINE" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="KABOLINE" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="KABOLINE" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
@@ -238,53 +238,53 @@
     <definedName name="KABOLINE" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="latent" localSheetId="7">#REF!</definedName>
     <definedName name="latent">'[4]steam table'!$N$5:$Q$102</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Break Down CI'!$7:$7</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Detailed PL'!$13:$14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Break Down CI'!$7:$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Detailed PL'!$13:$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'PL(2_2)'!$13:$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Technical Description'!$7:$8</definedName>
     <definedName name="SM" localSheetId="5" hidden="1">#REF!</definedName>
     <definedName name="SM" localSheetId="6" hidden="1">#REF!</definedName>
     <definedName name="SM" hidden="1">#REF!</definedName>
     <definedName name="tube_test_press1_12">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Break Down CI'!$A$1:$M$12</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Commercial Invoice'!$A$1:$K$47</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Detailed PL'!$A$1:$U$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Break Down CI'!$A$1:$O$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Commercial Invoice'!$A$1:$K$47</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Detailed PL'!$A$1:$U$19</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Packing List (1_2)'!$A$1:$K$48</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'PL(2_2)'!$B$1:$T$17</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'SHIPPING MARK (001)'!$A$1:$J$24</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'SHIPPING MARK (2)'!$A$1:$J$24</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Technical Description'!$A$1:$H$11</definedName>
+    <definedName name="weki_9701.xls" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="weki_9701.xls" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="weki_9701.xls" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="weki_9701.xls" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="weki_9701.xls" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="weki_9701.xls" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="weki_9701.xls" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="weki_9701.xls" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="wekir9701.xls" localSheetId="0" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="wekir9701.xls" localSheetId="2" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="wekir9701.xls" localSheetId="1" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="wekir9701.xls" localSheetId="3" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="wekir9701.xls" localSheetId="5" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="wekir9701.xls" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="wekir9701.xls" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="wekir9701.xls" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="X" localSheetId="0" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="X" localSheetId="2" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="X" localSheetId="1" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="X" localSheetId="3" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="X" localSheetId="5" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="X" localSheetId="6" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="X" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="X" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="Z" localSheetId="0" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="Z" localSheetId="2" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="Z" localSheetId="1" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="Z" localSheetId="3" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="Z" localSheetId="5" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="Z" localSheetId="6" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="Z" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="Z" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="ㄴㅇㄹㅇㄹ" localSheetId="0" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㄴㅇㄹㅇㄹ" localSheetId="2" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㄴㅇㄹㅇㄹ" localSheetId="1" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="ㄴㅇㄹㅇㄹ" localSheetId="0" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㄴㅇㄹㅇㄹ" localSheetId="3" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㄴㅇㄹㅇㄹ" localSheetId="5" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㄴㅇㄹㅇㄹ" localSheetId="6" hidden="1">'[2]Eq. Mobilization'!#REF!</definedName>
@@ -294,73 +294,73 @@
     <definedName name="느" localSheetId="6" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
     <definedName name="느" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="느" hidden="1">'[1]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="ㅊㅌㅍㅊㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍ" localSheetId="2" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍ" localSheetId="1" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="ㅊㅌㅍㅊㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍ" localSheetId="3" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍ" localSheetId="5" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍ" localSheetId="6" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍ" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍㅊㅌㅍ" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="ㅊㅌㅍㅊㅍㅌㅋㅊㅍㅌㅊㅍ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅌㅋㅊㅍㅌㅊㅍ" localSheetId="2" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅌㅋㅊㅍㅌㅊㅍ" localSheetId="1" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="ㅊㅌㅍㅊㅍㅌㅋㅊㅍㅌㅊㅍ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅌㅋㅊㅍㅌㅊㅍ" localSheetId="3" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅌㅋㅊㅍㅌㅊㅍ" localSheetId="5" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅌㅋㅊㅍㅌㅊㅍ" localSheetId="6" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅌㅋㅊㅍㅌㅊㅍ" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="ㅊㅌㅍㅊㅍㅌㅋㅊㅍㅌㅊㅍ" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="ㅊㅌㅍㅋㅊㅍㅌㅊㅍㅌㅊㅍ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅋㅊㅍㅌㅊㅍㅌㅊㅍ" localSheetId="2" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅋㅊㅍㅌㅊㅍㅌㅊㅍ" localSheetId="1" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="ㅊㅌㅍㅋㅊㅍㅌㅊㅍㅌㅊㅍ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅋㅊㅍㅌㅊㅍㅌㅊㅍ" localSheetId="3" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅋㅊㅍㅌㅊㅍㅌㅊㅍ" localSheetId="5" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅋㅊㅍㅌㅊㅍㅌㅊㅍ" localSheetId="6" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅋㅊㅍㅌㅊㅍㅌㅊㅍ" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="ㅊㅌㅍㅋㅊㅍㅌㅊㅍㅌㅊㅍ" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="ㅊㅌㅍㅌㅊㅍㅊㅌㅍㅌㅊㅍㅌㅊㅍ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅌㅊㅍㅊㅌㅍㅌㅊㅍㅌㅊㅍ" localSheetId="2" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅌㅊㅍㅊㅌㅍㅌㅊㅍㅌㅊㅍ" localSheetId="1" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="ㅊㅌㅍㅌㅊㅍㅊㅌㅍㅌㅊㅍㅌㅊㅍ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅌㅊㅍㅊㅌㅍㅌㅊㅍㅌㅊㅍ" localSheetId="3" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅌㅊㅍㅊㅌㅍㅌㅊㅍㅌㅊㅍ" localSheetId="5" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅌㅊㅍㅊㅌㅍㅌㅊㅍㅌㅊㅍ" localSheetId="6" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅊㅌㅍㅌㅊㅍㅊㅌㅍㅌㅊㅍㅌㅊㅍ" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="ㅊㅌㅍㅌㅊㅍㅊㅌㅍㅌㅊㅍㅌㅊㅍ" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="ㅋ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋ" localSheetId="2" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋ" localSheetId="1" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="ㅋ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋ" localSheetId="3" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋ" localSheetId="5" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋ" localSheetId="6" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋ" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="ㅋ" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="ㅋㅋㅋㅋ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋ" localSheetId="2" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋ" localSheetId="1" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="ㅋㅋㅋㅋ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋ" localSheetId="3" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋ" localSheetId="5" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋ" localSheetId="6" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋ" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋ" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="ㅋㅋㅋㅋㅋㅋ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋ" localSheetId="2" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋ" localSheetId="1" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="ㅋㅋㅋㅋㅋㅋ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋ" localSheetId="3" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋ" localSheetId="5" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋ" localSheetId="6" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋ" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋ" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="ㅋㅋㅋㅋㅋㅋㅋㅋㅋ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋㅋㅋㅋ" localSheetId="2" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋㅋㅋㅋ" localSheetId="1" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="ㅋㅋㅋㅋㅋㅋㅋㅋㅋ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋㅋㅋㅋ" localSheetId="3" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋㅋㅋㅋ" localSheetId="5" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋㅋㅋㅋ" localSheetId="6" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋㅋㅋㅋ" localSheetId="7" hidden="1">#REF!</definedName>
     <definedName name="ㅋㅋㅋㅋㅋㅋㅋㅋㅋ" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
+    <definedName name="ㅌㅊㅍㅌㅊㅍㅌㅋㅊㅍㅌ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅌㅊㅍㅌㅊㅍㅌㅋㅊㅍㅌ" localSheetId="2" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅌㅊㅍㅌㅊㅍㅌㅋㅊㅍㅌ" localSheetId="1" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
-    <definedName name="ㅌㅊㅍㅌㅊㅍㅌㅋㅊㅍㅌ" localSheetId="0" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅌㅊㅍㅌㅊㅍㅌㅋㅊㅍㅌ" localSheetId="3" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅌㅊㅍㅌㅊㅍㅌㅋㅊㅍㅌ" localSheetId="5" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
     <definedName name="ㅌㅊㅍㅌㅊㅍㅌㅋㅊㅍㅌ" localSheetId="6" hidden="1">'[5]Eq. Mobilization'!#REF!</definedName>
@@ -388,7 +388,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="217">
   <si>
     <t>PECC2 Innovation Hub, 45 Street No.2, Truong Tho Ward, Thu Duc City, HCMC, Vietnam
 Tel: +84-28-2221 6468 | Fax: +84-28-2221 0408</t>
@@ -1418,6 +1418,15 @@
   <si>
     <t>Conduit &amp; Accessories included I&amp;C Conduit  (Zinc Primer Paint)</t>
     <phoneticPr fontId="34" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vị trí</t>
+  </si>
+  <si>
+    <t>Ngày Nhận</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Office </t>
   </si>
 </sst>
 </file>
@@ -2387,7 +2396,7 @@
     </xf>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="526">
+  <cellXfs count="530">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3493,10 +3502,454 @@
     <xf numFmtId="177" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="30" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="28" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="31" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="41" fontId="41" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="41" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="41" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="41" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="41" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="41" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="41" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="41" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="8" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="41" fontId="2" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="2" fillId="2" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="2" fillId="2" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="15" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="14" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="14" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="14" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="6" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="7" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="10" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="10" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="11" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="37" fontId="58" fillId="2" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3529,443 +3982,11 @@
     <xf numFmtId="0" fontId="47" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="41" fontId="2" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="2" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="2" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="2" fillId="2" borderId="7" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="2" fillId="2" borderId="20" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="41" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="41" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="41" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="41" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="41" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="41" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="41" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="41" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="41" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="37" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="15" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="30" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="28" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="31" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="14" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="14" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="14" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="6" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="7" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="10" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="10" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="11" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="37" fontId="58" fillId="2" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="14">
@@ -4003,6 +4024,126 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>402</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>108912</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>455532</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F8AEE470-DCE2-4D18-881B-F891B5EF8496}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2415942" y="108912"/>
+          <a:ext cx="5141430" cy="474018"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ko-KR" sz="1600" b="1" u="sng"/>
+            <a:t>BREAK DOWN of COMMERCIAL INVOICE</a:t>
+          </a:r>
+          <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1600" b="1" u="sng"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>177800</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>514350</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>70080</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="그림 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7CF006AE-F715-0CFA-8C16-7FB6CAE2FA8A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="177800" y="0"/>
+          <a:ext cx="6280150" cy="8909280"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -4111,56 +4252,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>177800</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>514350</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>70080</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="그림 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7CF006AE-F715-0CFA-8C16-7FB6CAE2FA8A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="177800" y="0"/>
-          <a:ext cx="6280150" cy="8909280"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -4308,77 +4400,6 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>402</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>108912</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>455532</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="TextBox 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F8AEE470-DCE2-4D18-881B-F891B5EF8496}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2415942" y="108912"/>
-          <a:ext cx="5141430" cy="474018"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" altLang="ko-KR" sz="1600" b="1" u="sng"/>
-            <a:t>BREAK DOWN of COMMERCIAL INVOICE</a:t>
-          </a:r>
-          <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1600" b="1" u="sng"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -9547,6 +9568,450 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FFFFC000"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A5:R26"/>
+  <sheetFormatPr defaultColWidth="8.76953125" defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="8.76953125" style="73"/>
+    <col min="2" max="2" width="16.72265625" style="73" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16.72265625" style="73" customWidth="1"/>
+    <col min="5" max="5" width="40.2265625" style="73" customWidth="1"/>
+    <col min="6" max="6" width="20.11328125" style="73" customWidth="1"/>
+    <col min="7" max="7" width="11.34375" style="73" customWidth="1"/>
+    <col min="8" max="8" width="8.06640625" style="73" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.41796875" style="73" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.703125" style="73" customWidth="1"/>
+    <col min="11" max="12" width="8.06640625" style="78" customWidth="1"/>
+    <col min="13" max="13" width="9.23828125" style="73" customWidth="1"/>
+    <col min="14" max="14" width="11.92578125" style="73" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.796875" style="73" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.875" style="73" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.00390625" style="73" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.86328125" style="73" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="8.76953125" style="73"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="1:18">
+      <c r="B5" s="74" t="str">
+        <f>'Commercial Invoice'!G5</f>
+        <v>INVOICE NO. :</v>
+      </c>
+      <c r="C5" s="74"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="74" t="str">
+        <f>'Commercial Invoice'!H5</f>
+        <v>OM4-DE-IS-0010</v>
+      </c>
+      <c r="F5" s="74"/>
+      <c r="G5" s="75"/>
+      <c r="H5" s="74"/>
+      <c r="I5" s="74"/>
+      <c r="J5" s="74"/>
+      <c r="K5" s="446"/>
+      <c r="L5" s="447"/>
+      <c r="M5" s="76" t="s">
+        <v>127</v>
+      </c>
+      <c r="N5" s="76"/>
+      <c r="O5" s="191">
+        <f>'Commercial Invoice'!H6</f>
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18">
+      <c r="B6" s="77"/>
+      <c r="C6" s="77"/>
+      <c r="D6" s="77"/>
+      <c r="E6" s="77"/>
+      <c r="F6" s="77"/>
+    </row>
+    <row r="7" spans="1:18" ht="47.25" customHeight="1">
+      <c r="A7" s="448" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="450" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="368" t="s">
+        <v>214</v>
+      </c>
+      <c r="D7" s="368" t="s">
+        <v>215</v>
+      </c>
+      <c r="E7" s="452" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="450" t="s">
+        <v>152</v>
+      </c>
+      <c r="G7" s="448" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" s="454" t="s">
+        <v>153</v>
+      </c>
+      <c r="I7" s="455"/>
+      <c r="J7" s="448" t="s">
+        <v>154</v>
+      </c>
+      <c r="K7" s="448" t="s">
+        <v>161</v>
+      </c>
+      <c r="L7" s="448" t="s">
+        <v>160</v>
+      </c>
+      <c r="M7" s="448" t="s">
+        <v>155</v>
+      </c>
+      <c r="N7" s="448" t="s">
+        <v>156</v>
+      </c>
+      <c r="O7" s="452" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="14.45" customHeight="1">
+      <c r="A8" s="449"/>
+      <c r="B8" s="451"/>
+      <c r="C8" s="369"/>
+      <c r="D8" s="369"/>
+      <c r="E8" s="453"/>
+      <c r="F8" s="451"/>
+      <c r="G8" s="449"/>
+      <c r="H8" s="200" t="s">
+        <v>158</v>
+      </c>
+      <c r="I8" s="200" t="s">
+        <v>159</v>
+      </c>
+      <c r="J8" s="449"/>
+      <c r="K8" s="449"/>
+      <c r="L8" s="449"/>
+      <c r="M8" s="449"/>
+      <c r="N8" s="449"/>
+      <c r="O8" s="453"/>
+      <c r="Q8" s="73" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="14.45" customHeight="1">
+      <c r="A9" s="262">
+        <v>1</v>
+      </c>
+      <c r="B9" s="290" t="s">
+        <v>201</v>
+      </c>
+      <c r="C9" s="528" t="s">
+        <v>216</v>
+      </c>
+      <c r="D9" s="529">
+        <v>46231</v>
+      </c>
+      <c r="E9" s="349" t="s">
+        <v>205</v>
+      </c>
+      <c r="F9" s="268" t="s">
+        <v>163</v>
+      </c>
+      <c r="G9" s="290" t="s">
+        <v>198</v>
+      </c>
+      <c r="H9" s="350">
+        <f>'Detailed PL'!I15</f>
+        <v>32</v>
+      </c>
+      <c r="I9" s="351" t="str">
+        <f>'Detailed PL'!J15</f>
+        <v>EA</v>
+      </c>
+      <c r="J9" s="351" t="str">
+        <f>'Detailed PL'!K16</f>
+        <v>Wooden</v>
+      </c>
+      <c r="K9" s="352">
+        <f>'Detailed PL'!P16</f>
+        <v>576</v>
+      </c>
+      <c r="L9" s="352">
+        <f>'Detailed PL'!Q16</f>
+        <v>726</v>
+      </c>
+      <c r="M9" s="270">
+        <v>90.67</v>
+      </c>
+      <c r="N9" s="270">
+        <v>2901.44</v>
+      </c>
+      <c r="O9" s="270" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q9" s="342" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="14.45" customHeight="1">
+      <c r="A10" s="262">
+        <v>2</v>
+      </c>
+      <c r="B10" s="290" t="s">
+        <v>206</v>
+      </c>
+      <c r="C10" s="528" t="s">
+        <v>216</v>
+      </c>
+      <c r="D10" s="529">
+        <v>46231</v>
+      </c>
+      <c r="E10" s="349" t="s">
+        <v>205</v>
+      </c>
+      <c r="F10" s="268" t="s">
+        <v>163</v>
+      </c>
+      <c r="G10" s="290" t="s">
+        <v>198</v>
+      </c>
+      <c r="H10" s="350">
+        <f>'Detailed PL'!I17</f>
+        <v>18</v>
+      </c>
+      <c r="I10" s="351" t="str">
+        <f>'Detailed PL'!J17</f>
+        <v>EA</v>
+      </c>
+      <c r="J10" s="351" t="str">
+        <f>'Detailed PL'!K18</f>
+        <v>Wooden</v>
+      </c>
+      <c r="K10" s="352">
+        <f>'Detailed PL'!P18</f>
+        <v>324</v>
+      </c>
+      <c r="L10" s="352">
+        <f>'Detailed PL'!Q18</f>
+        <v>474</v>
+      </c>
+      <c r="M10" s="270">
+        <v>90.68</v>
+      </c>
+      <c r="N10" s="270">
+        <v>1632.23</v>
+      </c>
+      <c r="O10" s="270" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q10" s="342" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="14.1" customHeight="1">
+      <c r="A11" s="82"/>
+      <c r="B11" s="83"/>
+      <c r="C11" s="84"/>
+      <c r="D11" s="84"/>
+      <c r="E11" s="84"/>
+      <c r="F11" s="84"/>
+      <c r="G11" s="85"/>
+      <c r="H11" s="86"/>
+      <c r="I11" s="86"/>
+      <c r="J11" s="87" t="s">
+        <v>32</v>
+      </c>
+      <c r="K11" s="88"/>
+      <c r="L11" s="84"/>
+      <c r="M11" s="84"/>
+      <c r="N11" s="327">
+        <f>SUM(N9:N10)</f>
+        <v>4533.67</v>
+      </c>
+      <c r="O11" s="89"/>
+      <c r="Q11" s="343"/>
+      <c r="R11" s="342"/>
+    </row>
+    <row r="12" spans="1:18" ht="14.1" customHeight="1">
+      <c r="A12" s="90"/>
+      <c r="B12" s="91"/>
+      <c r="C12" s="81"/>
+      <c r="D12" s="81"/>
+      <c r="E12" s="81"/>
+      <c r="F12" s="81"/>
+      <c r="G12" s="92"/>
+      <c r="H12" s="93"/>
+      <c r="I12" s="93"/>
+      <c r="J12" s="93"/>
+      <c r="K12" s="94"/>
+      <c r="L12" s="94"/>
+      <c r="M12" s="81"/>
+      <c r="N12" s="81"/>
+      <c r="O12" s="91"/>
+      <c r="P12" s="80"/>
+      <c r="Q12" s="80">
+        <f>N9+P19</f>
+        <v>5802.88</v>
+      </c>
+      <c r="R12" s="346"/>
+    </row>
+    <row r="13" spans="1:18">
+      <c r="Q13" s="80">
+        <f>N10+P20</f>
+        <v>3264.4700000000003</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18">
+      <c r="P14" s="346"/>
+      <c r="Q14" s="346"/>
+      <c r="R14" s="80"/>
+    </row>
+    <row r="15" spans="1:18">
+      <c r="P15" s="346"/>
+      <c r="Q15" s="346"/>
+      <c r="R15" s="80"/>
+    </row>
+    <row r="16" spans="1:18">
+      <c r="N16" s="353">
+        <f>M9*H9</f>
+        <v>2901.44</v>
+      </c>
+      <c r="P16" s="346">
+        <f>H9*M9</f>
+        <v>2901.44</v>
+      </c>
+    </row>
+    <row r="17" spans="13:18">
+      <c r="N17" s="353">
+        <f>M10*H10</f>
+        <v>1632.2400000000002</v>
+      </c>
+      <c r="P17" s="346">
+        <f>H10*M10</f>
+        <v>1632.2400000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="13:18">
+      <c r="M18" s="342"/>
+      <c r="N18" s="353">
+        <f>SUM(N16:N17)</f>
+        <v>4533.68</v>
+      </c>
+      <c r="P18" s="80"/>
+    </row>
+    <row r="19" spans="13:18">
+      <c r="M19" s="342"/>
+      <c r="N19" s="78"/>
+      <c r="P19" s="80">
+        <f>ROUND(P16,2)</f>
+        <v>2901.44</v>
+      </c>
+    </row>
+    <row r="20" spans="13:18">
+      <c r="M20" s="342"/>
+      <c r="N20" s="73">
+        <v>2901.55</v>
+      </c>
+      <c r="P20" s="80">
+        <f>ROUND(P17,2)</f>
+        <v>1632.24</v>
+      </c>
+      <c r="R20" s="356"/>
+    </row>
+    <row r="21" spans="13:18">
+      <c r="M21" s="342"/>
+      <c r="N21" s="73">
+        <v>1632.12</v>
+      </c>
+    </row>
+    <row r="22" spans="13:18">
+      <c r="N22" s="73">
+        <v>4533.67</v>
+      </c>
+    </row>
+    <row r="25" spans="13:18">
+      <c r="O25" s="346"/>
+    </row>
+    <row r="26" spans="13:18">
+      <c r="P26" s="367"/>
+      <c r="Q26" s="367"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:P11" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <mergeCells count="13">
+    <mergeCell ref="M7:M8"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="G7:G8"/>
+  </mergeCells>
+  <phoneticPr fontId="34" type="noConversion"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.70866141732283472" right="0.31496062992125984" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="67" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FF0070C0"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetData/>
+  <phoneticPr fontId="34" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FF002060"/>
+  </sheetPr>
+  <dimension ref="I3"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
+  <cols>
+    <col min="9" max="9" width="80.80859375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="9:9" ht="57">
+      <c r="I3" s="175" t="s">
+        <v>112</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="34" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <dimension ref="A2"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetData>
+    <row r="2" ht="24" customHeight="1"/>
+  </sheetData>
+  <phoneticPr fontId="34" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor rgb="FF92D050"/>
@@ -9583,26 +10048,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:40" ht="9" customHeight="1">
-      <c r="B1" s="369"/>
-      <c r="C1" s="369"/>
-      <c r="D1" s="369"/>
-      <c r="E1" s="369"/>
-      <c r="F1" s="369"/>
-      <c r="G1" s="369"/>
-      <c r="H1" s="369"/>
-      <c r="I1" s="369"/>
-      <c r="J1" s="369"/>
-      <c r="K1" s="369"/>
-      <c r="L1" s="369"/>
-      <c r="M1" s="369"/>
-      <c r="N1" s="369"/>
-      <c r="O1" s="369"/>
-      <c r="P1" s="369"/>
-      <c r="Q1" s="369"/>
-      <c r="R1" s="369"/>
-      <c r="S1" s="369"/>
-      <c r="T1" s="369"/>
-      <c r="U1" s="369"/>
+      <c r="B1" s="376"/>
+      <c r="C1" s="376"/>
+      <c r="D1" s="376"/>
+      <c r="E1" s="376"/>
+      <c r="F1" s="376"/>
+      <c r="G1" s="376"/>
+      <c r="H1" s="376"/>
+      <c r="I1" s="376"/>
+      <c r="J1" s="376"/>
+      <c r="K1" s="376"/>
+      <c r="L1" s="376"/>
+      <c r="M1" s="376"/>
+      <c r="N1" s="376"/>
+      <c r="O1" s="376"/>
+      <c r="P1" s="376"/>
+      <c r="Q1" s="376"/>
+      <c r="R1" s="376"/>
+      <c r="S1" s="376"/>
+      <c r="T1" s="376"/>
+      <c r="U1" s="376"/>
     </row>
     <row r="2" spans="2:40" ht="26.1" customHeight="1">
       <c r="B2" s="133"/>
@@ -9640,17 +10105,17 @@
     </row>
     <row r="3" spans="2:40" ht="27.6" customHeight="1" thickBot="1">
       <c r="B3" s="133"/>
-      <c r="C3" s="490" t="s">
+      <c r="C3" s="377" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="490"/>
-      <c r="E3" s="490"/>
-      <c r="F3" s="490"/>
-      <c r="G3" s="490"/>
-      <c r="H3" s="490"/>
-      <c r="I3" s="490"/>
-      <c r="J3" s="490"/>
-      <c r="K3" s="490"/>
+      <c r="D3" s="377"/>
+      <c r="E3" s="377"/>
+      <c r="F3" s="377"/>
+      <c r="G3" s="377"/>
+      <c r="H3" s="377"/>
+      <c r="I3" s="377"/>
+      <c r="J3" s="377"/>
+      <c r="K3" s="377"/>
       <c r="L3" s="137"/>
       <c r="M3" s="138"/>
       <c r="N3" s="139"/>
@@ -9676,28 +10141,28 @@
       <c r="AN3" s="136"/>
     </row>
     <row r="4" spans="2:40" ht="33.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B4" s="491" t="s">
+      <c r="B4" s="378" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="492"/>
-      <c r="D4" s="492"/>
-      <c r="E4" s="492"/>
-      <c r="F4" s="492"/>
-      <c r="G4" s="492"/>
-      <c r="H4" s="492"/>
-      <c r="I4" s="492"/>
-      <c r="J4" s="492"/>
-      <c r="K4" s="492"/>
-      <c r="L4" s="492"/>
-      <c r="M4" s="492"/>
-      <c r="N4" s="492"/>
-      <c r="O4" s="492"/>
-      <c r="P4" s="492"/>
-      <c r="Q4" s="492"/>
-      <c r="R4" s="492"/>
-      <c r="S4" s="492"/>
-      <c r="T4" s="492"/>
-      <c r="U4" s="493"/>
+      <c r="C4" s="379"/>
+      <c r="D4" s="379"/>
+      <c r="E4" s="379"/>
+      <c r="F4" s="379"/>
+      <c r="G4" s="379"/>
+      <c r="H4" s="379"/>
+      <c r="I4" s="379"/>
+      <c r="J4" s="379"/>
+      <c r="K4" s="379"/>
+      <c r="L4" s="379"/>
+      <c r="M4" s="379"/>
+      <c r="N4" s="379"/>
+      <c r="O4" s="379"/>
+      <c r="P4" s="379"/>
+      <c r="Q4" s="379"/>
+      <c r="R4" s="379"/>
+      <c r="S4" s="379"/>
+      <c r="T4" s="379"/>
+      <c r="U4" s="380"/>
     </row>
     <row r="5" spans="2:40" s="73" customFormat="1" ht="17.25" customHeight="1" thickTop="1">
       <c r="B5" s="78"/>
@@ -10037,54 +10502,54 @@
       <c r="AN12" s="78"/>
     </row>
     <row r="13" spans="2:40" s="152" customFormat="1" ht="20.25" customHeight="1">
-      <c r="B13" s="494" t="s">
+      <c r="B13" s="371" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="496" t="s">
+      <c r="C13" s="382" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="497" t="s">
+      <c r="D13" s="383" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="498"/>
-      <c r="F13" s="494" t="s">
+      <c r="E13" s="384"/>
+      <c r="F13" s="371" t="s">
         <v>90</v>
       </c>
-      <c r="G13" s="496" t="s">
+      <c r="G13" s="382" t="s">
         <v>144</v>
       </c>
-      <c r="H13" s="494" t="s">
+      <c r="H13" s="371" t="s">
         <v>145</v>
       </c>
-      <c r="I13" s="502" t="s">
+      <c r="I13" s="387" t="s">
         <v>72</v>
       </c>
-      <c r="J13" s="503"/>
-      <c r="K13" s="494" t="s">
+      <c r="J13" s="388"/>
+      <c r="K13" s="371" t="s">
         <v>73</v>
       </c>
-      <c r="L13" s="502" t="s">
+      <c r="L13" s="387" t="s">
         <v>74</v>
       </c>
-      <c r="M13" s="504"/>
-      <c r="N13" s="504"/>
-      <c r="O13" s="503"/>
-      <c r="P13" s="494" t="s">
+      <c r="M13" s="389"/>
+      <c r="N13" s="389"/>
+      <c r="O13" s="388"/>
+      <c r="P13" s="371" t="s">
         <v>75</v>
       </c>
-      <c r="Q13" s="494" t="s">
+      <c r="Q13" s="371" t="s">
         <v>76</v>
       </c>
-      <c r="R13" s="494" t="s">
+      <c r="R13" s="371" t="s">
         <v>77</v>
       </c>
-      <c r="S13" s="494" t="s">
+      <c r="S13" s="371" t="s">
         <v>78</v>
       </c>
-      <c r="T13" s="497" t="s">
+      <c r="T13" s="383" t="s">
         <v>91</v>
       </c>
-      <c r="U13" s="494" t="s">
+      <c r="U13" s="371" t="s">
         <v>79</v>
       </c>
       <c r="V13" s="150"/>
@@ -10102,20 +10567,20 @@
       <c r="AN13" s="151"/>
     </row>
     <row r="14" spans="2:40" s="152" customFormat="1" ht="28.5" customHeight="1">
-      <c r="B14" s="495"/>
-      <c r="C14" s="495"/>
-      <c r="D14" s="499"/>
-      <c r="E14" s="500"/>
-      <c r="F14" s="501"/>
-      <c r="G14" s="495"/>
-      <c r="H14" s="501"/>
+      <c r="B14" s="381"/>
+      <c r="C14" s="381"/>
+      <c r="D14" s="385"/>
+      <c r="E14" s="386"/>
+      <c r="F14" s="372"/>
+      <c r="G14" s="381"/>
+      <c r="H14" s="372"/>
       <c r="I14" s="201" t="s">
         <v>80</v>
       </c>
       <c r="J14" s="153" t="s">
         <v>81</v>
       </c>
-      <c r="K14" s="501"/>
+      <c r="K14" s="372"/>
       <c r="L14" s="154" t="s">
         <v>82</v>
       </c>
@@ -10128,12 +10593,12 @@
       <c r="O14" s="155" t="s">
         <v>85</v>
       </c>
-      <c r="P14" s="501"/>
-      <c r="Q14" s="501"/>
-      <c r="R14" s="501"/>
-      <c r="S14" s="501"/>
-      <c r="T14" s="499"/>
-      <c r="U14" s="501"/>
+      <c r="P14" s="372"/>
+      <c r="Q14" s="372"/>
+      <c r="R14" s="372"/>
+      <c r="S14" s="372"/>
+      <c r="T14" s="385"/>
+      <c r="U14" s="372"/>
       <c r="W14" s="151"/>
       <c r="X14" s="151"/>
       <c r="Y14" s="151"/>
@@ -10202,15 +10667,15 @@
       <c r="AN15" s="151"/>
     </row>
     <row r="16" spans="2:40" s="152" customFormat="1" ht="28.5" customHeight="1">
-      <c r="B16" s="506" t="s">
+      <c r="B16" s="373" t="s">
         <v>92</v>
       </c>
-      <c r="C16" s="507"/>
-      <c r="D16" s="507"/>
-      <c r="E16" s="507"/>
-      <c r="F16" s="507"/>
-      <c r="G16" s="507"/>
-      <c r="H16" s="508"/>
+      <c r="C16" s="374"/>
+      <c r="D16" s="374"/>
+      <c r="E16" s="374"/>
+      <c r="F16" s="374"/>
+      <c r="G16" s="374"/>
+      <c r="H16" s="375"/>
       <c r="I16" s="255">
         <f>SUM(I15)</f>
         <v>32</v>
@@ -10317,15 +10782,15 @@
       <c r="AN17" s="151"/>
     </row>
     <row r="18" spans="2:40" s="152" customFormat="1" ht="28.5" customHeight="1">
-      <c r="B18" s="506" t="s">
+      <c r="B18" s="373" t="s">
         <v>92</v>
       </c>
-      <c r="C18" s="507"/>
-      <c r="D18" s="507"/>
-      <c r="E18" s="507"/>
-      <c r="F18" s="507"/>
-      <c r="G18" s="507"/>
-      <c r="H18" s="508"/>
+      <c r="C18" s="374"/>
+      <c r="D18" s="374"/>
+      <c r="E18" s="374"/>
+      <c r="F18" s="374"/>
+      <c r="G18" s="374"/>
+      <c r="H18" s="375"/>
       <c r="I18" s="255">
         <f>SUM(I17:I17)</f>
         <v>18</v>
@@ -10378,17 +10843,17 @@
       <c r="AN18" s="151"/>
     </row>
     <row r="19" spans="2:40" s="73" customFormat="1" ht="32.25" customHeight="1">
-      <c r="B19" s="505" t="s">
+      <c r="B19" s="370" t="s">
         <v>93</v>
       </c>
-      <c r="C19" s="505"/>
-      <c r="D19" s="505"/>
-      <c r="E19" s="505"/>
-      <c r="F19" s="505"/>
-      <c r="G19" s="505"/>
-      <c r="H19" s="505"/>
-      <c r="I19" s="505"/>
-      <c r="J19" s="505"/>
+      <c r="C19" s="370"/>
+      <c r="D19" s="370"/>
+      <c r="E19" s="370"/>
+      <c r="F19" s="370"/>
+      <c r="G19" s="370"/>
+      <c r="H19" s="370"/>
+      <c r="I19" s="370"/>
+      <c r="J19" s="370"/>
       <c r="K19" s="79"/>
       <c r="L19" s="79"/>
       <c r="M19" s="79"/>
@@ -10428,13 +10893,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B19:J19"/>
-    <mergeCell ref="P13:P14"/>
-    <mergeCell ref="Q13:Q14"/>
-    <mergeCell ref="R13:R14"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="B18:H18"/>
     <mergeCell ref="B1:U1"/>
     <mergeCell ref="C3:K3"/>
     <mergeCell ref="B4:U4"/>
@@ -10449,6 +10907,13 @@
     <mergeCell ref="S13:S14"/>
     <mergeCell ref="T13:T14"/>
     <mergeCell ref="G13:G14"/>
+    <mergeCell ref="B19:J19"/>
+    <mergeCell ref="P13:P14"/>
+    <mergeCell ref="Q13:Q14"/>
+    <mergeCell ref="R13:R14"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B18:H18"/>
   </mergeCells>
   <phoneticPr fontId="34" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -10461,57 +10926,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <sheetPr>
-    <tabColor rgb="FF0070C0"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
-  <sheetData/>
-  <phoneticPr fontId="34" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <sheetPr>
-    <tabColor rgb="FF002060"/>
-  </sheetPr>
-  <dimension ref="I3"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
-  <cols>
-    <col min="9" max="9" width="80.80859375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="9:9" ht="57">
-      <c r="I3" s="175" t="s">
-        <v>112</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="34" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A2"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
-  <sheetData>
-    <row r="2" ht="24" customHeight="1"/>
-  </sheetData>
-  <phoneticPr fontId="34" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
@@ -10562,33 +10977,33 @@
     </row>
     <row r="3" spans="1:14" ht="37.5" customHeight="1">
       <c r="A3" s="10"/>
-      <c r="B3" s="422" t="s">
+      <c r="B3" s="390" t="s">
         <v>114</v>
       </c>
-      <c r="C3" s="423"/>
-      <c r="D3" s="423"/>
-      <c r="E3" s="423"/>
+      <c r="C3" s="391"/>
+      <c r="D3" s="391"/>
+      <c r="E3" s="391"/>
       <c r="F3" s="183"/>
       <c r="G3" s="184"/>
-      <c r="H3" s="422"/>
-      <c r="I3" s="423"/>
-      <c r="J3" s="423"/>
-      <c r="K3" s="424"/>
+      <c r="H3" s="390"/>
+      <c r="I3" s="391"/>
+      <c r="J3" s="391"/>
+      <c r="K3" s="392"/>
     </row>
     <row r="4" spans="1:14" s="13" customFormat="1" ht="24.75" customHeight="1">
-      <c r="A4" s="425" t="s">
+      <c r="A4" s="393" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="426"/>
-      <c r="C4" s="426"/>
-      <c r="D4" s="426"/>
-      <c r="E4" s="426"/>
-      <c r="F4" s="426"/>
-      <c r="G4" s="426"/>
-      <c r="H4" s="426"/>
-      <c r="I4" s="426"/>
-      <c r="J4" s="426"/>
-      <c r="K4" s="427"/>
+      <c r="B4" s="394"/>
+      <c r="C4" s="394"/>
+      <c r="D4" s="394"/>
+      <c r="E4" s="394"/>
+      <c r="F4" s="394"/>
+      <c r="G4" s="394"/>
+      <c r="H4" s="394"/>
+      <c r="I4" s="394"/>
+      <c r="J4" s="394"/>
+      <c r="K4" s="395"/>
       <c r="L4" s="11"/>
       <c r="M4" s="12"/>
       <c r="N4" s="12"/>
@@ -10617,13 +11032,13 @@
     </row>
     <row r="6" spans="1:14" s="13" customFormat="1" ht="12.75">
       <c r="A6" s="23"/>
-      <c r="B6" s="431" t="s">
+      <c r="B6" s="399" t="s">
         <v>130</v>
       </c>
-      <c r="C6" s="432"/>
-      <c r="D6" s="432"/>
-      <c r="E6" s="432"/>
-      <c r="F6" s="433"/>
+      <c r="C6" s="400"/>
+      <c r="D6" s="400"/>
+      <c r="E6" s="400"/>
+      <c r="F6" s="401"/>
       <c r="G6" s="24" t="s">
         <v>4</v>
       </c>
@@ -10639,11 +11054,11 @@
     </row>
     <row r="7" spans="1:14" ht="15.4" customHeight="1">
       <c r="A7" s="8"/>
-      <c r="B7" s="432"/>
-      <c r="C7" s="432"/>
-      <c r="D7" s="432"/>
-      <c r="E7" s="432"/>
-      <c r="F7" s="433"/>
+      <c r="B7" s="400"/>
+      <c r="C7" s="400"/>
+      <c r="D7" s="400"/>
+      <c r="E7" s="400"/>
+      <c r="F7" s="401"/>
       <c r="G7" s="29" t="s">
         <v>5</v>
       </c>
@@ -10656,11 +11071,11 @@
     </row>
     <row r="8" spans="1:14" ht="16.5" customHeight="1">
       <c r="A8" s="8"/>
-      <c r="B8" s="434"/>
-      <c r="C8" s="434"/>
-      <c r="D8" s="434"/>
-      <c r="E8" s="434"/>
-      <c r="F8" s="435"/>
+      <c r="B8" s="402"/>
+      <c r="C8" s="402"/>
+      <c r="D8" s="402"/>
+      <c r="E8" s="402"/>
+      <c r="F8" s="403"/>
       <c r="G8" s="24" t="s">
         <v>4</v>
       </c>
@@ -10680,56 +11095,56 @@
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
       <c r="F9" s="34"/>
-      <c r="G9" s="428" t="s">
+      <c r="G9" s="396" t="s">
         <v>8</v>
       </c>
-      <c r="H9" s="429"/>
-      <c r="I9" s="429"/>
-      <c r="J9" s="429"/>
-      <c r="K9" s="430"/>
+      <c r="H9" s="397"/>
+      <c r="I9" s="397"/>
+      <c r="J9" s="397"/>
+      <c r="K9" s="398"/>
     </row>
     <row r="10" spans="1:14" ht="14.1" customHeight="1">
       <c r="A10" s="8"/>
-      <c r="B10" s="413" t="s">
+      <c r="B10" s="420" t="s">
         <v>129</v>
       </c>
-      <c r="C10" s="413"/>
-      <c r="D10" s="413"/>
-      <c r="E10" s="413"/>
-      <c r="F10" s="414"/>
-      <c r="G10" s="399" t="s">
+      <c r="C10" s="420"/>
+      <c r="D10" s="420"/>
+      <c r="E10" s="420"/>
+      <c r="F10" s="421"/>
+      <c r="G10" s="404" t="s">
         <v>126</v>
       </c>
-      <c r="H10" s="400"/>
-      <c r="I10" s="400"/>
-      <c r="J10" s="400"/>
-      <c r="K10" s="401"/>
+      <c r="H10" s="405"/>
+      <c r="I10" s="405"/>
+      <c r="J10" s="405"/>
+      <c r="K10" s="406"/>
     </row>
     <row r="11" spans="1:14" ht="14.1" customHeight="1">
       <c r="A11" s="8"/>
-      <c r="B11" s="413"/>
-      <c r="C11" s="413"/>
-      <c r="D11" s="413"/>
-      <c r="E11" s="413"/>
-      <c r="F11" s="414"/>
-      <c r="G11" s="402"/>
-      <c r="H11" s="403"/>
-      <c r="I11" s="403"/>
-      <c r="J11" s="403"/>
-      <c r="K11" s="404"/>
+      <c r="B11" s="420"/>
+      <c r="C11" s="420"/>
+      <c r="D11" s="420"/>
+      <c r="E11" s="420"/>
+      <c r="F11" s="421"/>
+      <c r="G11" s="407"/>
+      <c r="H11" s="408"/>
+      <c r="I11" s="408"/>
+      <c r="J11" s="408"/>
+      <c r="K11" s="409"/>
     </row>
     <row r="12" spans="1:14" ht="28.15" customHeight="1" thickBot="1">
       <c r="A12" s="35"/>
-      <c r="B12" s="415"/>
-      <c r="C12" s="415"/>
-      <c r="D12" s="415"/>
-      <c r="E12" s="415"/>
-      <c r="F12" s="416"/>
-      <c r="G12" s="405"/>
-      <c r="H12" s="406"/>
-      <c r="I12" s="406"/>
-      <c r="J12" s="406"/>
-      <c r="K12" s="407"/>
+      <c r="B12" s="422"/>
+      <c r="C12" s="422"/>
+      <c r="D12" s="422"/>
+      <c r="E12" s="422"/>
+      <c r="F12" s="423"/>
+      <c r="G12" s="410"/>
+      <c r="H12" s="411"/>
+      <c r="I12" s="411"/>
+      <c r="J12" s="411"/>
+      <c r="K12" s="412"/>
     </row>
     <row r="13" spans="1:14" ht="14.1" customHeight="1">
       <c r="A13" s="36" t="s">
@@ -10748,67 +11163,67 @@
     </row>
     <row r="14" spans="1:14" ht="14.1" customHeight="1">
       <c r="A14" s="8"/>
-      <c r="B14" s="417" t="s">
+      <c r="B14" s="424" t="s">
         <v>131</v>
       </c>
-      <c r="C14" s="418"/>
-      <c r="D14" s="418"/>
-      <c r="E14" s="418"/>
-      <c r="F14" s="419"/>
+      <c r="C14" s="425"/>
+      <c r="D14" s="425"/>
+      <c r="E14" s="425"/>
+      <c r="F14" s="426"/>
       <c r="G14" s="38"/>
-      <c r="H14" s="408"/>
-      <c r="I14" s="408"/>
-      <c r="J14" s="408"/>
-      <c r="K14" s="409"/>
+      <c r="H14" s="413"/>
+      <c r="I14" s="413"/>
+      <c r="J14" s="413"/>
+      <c r="K14" s="414"/>
     </row>
     <row r="15" spans="1:14" s="278" customFormat="1" ht="14.1" customHeight="1">
       <c r="A15" s="276"/>
-      <c r="B15" s="418"/>
-      <c r="C15" s="418"/>
-      <c r="D15" s="418"/>
-      <c r="E15" s="418"/>
-      <c r="F15" s="419"/>
+      <c r="B15" s="425"/>
+      <c r="C15" s="425"/>
+      <c r="D15" s="425"/>
+      <c r="E15" s="425"/>
+      <c r="F15" s="426"/>
       <c r="G15" s="274" t="s">
         <v>11</v>
       </c>
-      <c r="H15" s="410" t="str">
+      <c r="H15" s="415" t="str">
         <f>H5</f>
         <v>OM4-DE-IS-0010</v>
       </c>
-      <c r="I15" s="411"/>
-      <c r="J15" s="411"/>
-      <c r="K15" s="412"/>
+      <c r="I15" s="416"/>
+      <c r="J15" s="416"/>
+      <c r="K15" s="417"/>
       <c r="L15" s="277"/>
     </row>
     <row r="16" spans="1:14" ht="9" customHeight="1">
       <c r="A16" s="8"/>
-      <c r="B16" s="418"/>
-      <c r="C16" s="418"/>
-      <c r="D16" s="418"/>
-      <c r="E16" s="418"/>
-      <c r="F16" s="419"/>
+      <c r="B16" s="425"/>
+      <c r="C16" s="425"/>
+      <c r="D16" s="425"/>
+      <c r="E16" s="425"/>
+      <c r="F16" s="426"/>
       <c r="G16" s="38"/>
-      <c r="H16" s="411"/>
-      <c r="I16" s="411"/>
-      <c r="J16" s="411"/>
-      <c r="K16" s="412"/>
+      <c r="H16" s="416"/>
+      <c r="I16" s="416"/>
+      <c r="J16" s="416"/>
+      <c r="K16" s="417"/>
     </row>
     <row r="17" spans="1:15" ht="100.15" customHeight="1">
       <c r="A17" s="8"/>
-      <c r="B17" s="420"/>
-      <c r="C17" s="420"/>
-      <c r="D17" s="420"/>
-      <c r="E17" s="420"/>
-      <c r="F17" s="421"/>
+      <c r="B17" s="427"/>
+      <c r="C17" s="427"/>
+      <c r="D17" s="427"/>
+      <c r="E17" s="427"/>
+      <c r="F17" s="428"/>
       <c r="G17" s="274" t="s">
         <v>12</v>
       </c>
-      <c r="H17" s="387" t="s">
+      <c r="H17" s="418" t="s">
         <v>196</v>
       </c>
-      <c r="I17" s="387"/>
-      <c r="J17" s="387"/>
-      <c r="K17" s="388"/>
+      <c r="I17" s="418"/>
+      <c r="J17" s="418"/>
+      <c r="K17" s="419"/>
     </row>
     <row r="18" spans="1:15" ht="18.600000000000001" customHeight="1">
       <c r="A18" s="33" t="s">
@@ -10822,10 +11237,10 @@
       <c r="E18" s="30"/>
       <c r="F18" s="34"/>
       <c r="G18" s="37"/>
-      <c r="H18" s="381"/>
-      <c r="I18" s="381"/>
-      <c r="J18" s="381"/>
-      <c r="K18" s="382"/>
+      <c r="H18" s="430"/>
+      <c r="I18" s="430"/>
+      <c r="J18" s="430"/>
+      <c r="K18" s="431"/>
     </row>
     <row r="19" spans="1:15" s="6" customFormat="1" ht="11.65" customHeight="1">
       <c r="A19" s="35"/>
@@ -10833,20 +11248,20 @@
         <v>210</v>
       </c>
       <c r="C19" s="261"/>
-      <c r="D19" s="383">
+      <c r="D19" s="432">
         <v>46208</v>
       </c>
-      <c r="E19" s="383"/>
-      <c r="F19" s="384"/>
+      <c r="E19" s="432"/>
+      <c r="F19" s="433"/>
       <c r="G19" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="H19" s="381" t="s">
+      <c r="H19" s="430" t="s">
         <v>111</v>
       </c>
-      <c r="I19" s="381"/>
-      <c r="J19" s="381"/>
-      <c r="K19" s="382"/>
+      <c r="I19" s="430"/>
+      <c r="J19" s="430"/>
+      <c r="K19" s="431"/>
       <c r="M19" s="7"/>
       <c r="N19" s="7"/>
       <c r="O19" s="7"/>
@@ -10865,12 +11280,12 @@
       <c r="G20" s="280" t="s">
         <v>190</v>
       </c>
-      <c r="H20" s="387" t="s">
+      <c r="H20" s="418" t="s">
         <v>189</v>
       </c>
-      <c r="I20" s="387"/>
-      <c r="J20" s="387"/>
-      <c r="K20" s="388"/>
+      <c r="I20" s="418"/>
+      <c r="J20" s="418"/>
+      <c r="K20" s="419"/>
       <c r="M20" s="7"/>
       <c r="N20" s="7"/>
       <c r="O20" s="7"/>
@@ -10919,9 +11334,9 @@
       <c r="A23" s="35"/>
       <c r="B23" s="260"/>
       <c r="C23" s="261"/>
-      <c r="D23" s="389"/>
-      <c r="E23" s="389"/>
-      <c r="F23" s="390"/>
+      <c r="D23" s="436"/>
+      <c r="E23" s="436"/>
+      <c r="F23" s="437"/>
       <c r="G23" s="37"/>
       <c r="H23" s="181"/>
       <c r="I23" s="181"/>
@@ -10969,13 +11384,13 @@
     </row>
     <row r="26" spans="1:15" s="6" customFormat="1" ht="12.75">
       <c r="A26" s="35"/>
-      <c r="B26" s="391" t="s">
+      <c r="B26" s="438" t="s">
         <v>132</v>
       </c>
-      <c r="C26" s="391"/>
-      <c r="D26" s="391"/>
-      <c r="E26" s="391"/>
-      <c r="F26" s="392"/>
+      <c r="C26" s="438"/>
+      <c r="D26" s="438"/>
+      <c r="E26" s="438"/>
+      <c r="F26" s="439"/>
       <c r="G26" s="47"/>
       <c r="H26" s="48"/>
       <c r="I26" s="48"/>
@@ -10986,15 +11401,15 @@
       <c r="O26" s="7"/>
     </row>
     <row r="27" spans="1:15" ht="45" customHeight="1">
-      <c r="A27" s="393" t="s">
+      <c r="A27" s="440" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="386"/>
-      <c r="C27" s="386"/>
-      <c r="D27" s="386"/>
-      <c r="E27" s="386"/>
-      <c r="F27" s="386"/>
-      <c r="G27" s="394"/>
+      <c r="B27" s="435"/>
+      <c r="C27" s="435"/>
+      <c r="D27" s="435"/>
+      <c r="E27" s="435"/>
+      <c r="F27" s="435"/>
+      <c r="G27" s="441"/>
       <c r="H27" s="50" t="s">
         <v>21</v>
       </c>
@@ -11010,14 +11425,14 @@
     </row>
     <row r="28" spans="1:15" ht="36" customHeight="1">
       <c r="A28" s="36"/>
-      <c r="B28" s="395" t="s">
+      <c r="B28" s="442" t="s">
         <v>133</v>
       </c>
-      <c r="C28" s="395"/>
-      <c r="D28" s="395"/>
-      <c r="E28" s="395"/>
-      <c r="F28" s="395"/>
-      <c r="G28" s="396"/>
+      <c r="C28" s="442"/>
+      <c r="D28" s="442"/>
+      <c r="E28" s="442"/>
+      <c r="F28" s="442"/>
+      <c r="G28" s="443"/>
       <c r="H28" s="53"/>
       <c r="I28" s="53"/>
       <c r="J28" s="53"/>
@@ -11038,14 +11453,14 @@
     </row>
     <row r="30" spans="1:15" ht="15" customHeight="1">
       <c r="A30" s="263"/>
-      <c r="B30" s="397" t="s">
+      <c r="B30" s="444" t="s">
         <v>213</v>
       </c>
-      <c r="C30" s="397"/>
-      <c r="D30" s="397"/>
-      <c r="E30" s="397"/>
-      <c r="F30" s="397"/>
-      <c r="G30" s="398"/>
+      <c r="C30" s="444"/>
+      <c r="D30" s="444"/>
+      <c r="E30" s="444"/>
+      <c r="F30" s="444"/>
+      <c r="G30" s="445"/>
       <c r="H30" s="284" t="s">
         <v>146</v>
       </c>
@@ -11058,7 +11473,7 @@
         <v>90.67</v>
       </c>
       <c r="K30" s="295">
-        <f>'Break Down CI'!L9</f>
+        <f>'Break Down CI'!N9</f>
         <v>2901.44</v>
       </c>
       <c r="M30" s="311" t="s">
@@ -11067,12 +11482,12 @@
     </row>
     <row r="31" spans="1:15" ht="15" customHeight="1">
       <c r="A31" s="263"/>
-      <c r="B31" s="397"/>
-      <c r="C31" s="397"/>
-      <c r="D31" s="397"/>
-      <c r="E31" s="397"/>
-      <c r="F31" s="397"/>
-      <c r="G31" s="398"/>
+      <c r="B31" s="444"/>
+      <c r="C31" s="444"/>
+      <c r="D31" s="444"/>
+      <c r="E31" s="444"/>
+      <c r="F31" s="444"/>
+      <c r="G31" s="445"/>
       <c r="H31" s="284" t="s">
         <v>146</v>
       </c>
@@ -11085,7 +11500,7 @@
         <v>90.68</v>
       </c>
       <c r="K31" s="295">
-        <f>'Break Down CI'!L10</f>
+        <f>'Break Down CI'!N10</f>
         <v>1632.23</v>
       </c>
     </row>
@@ -11192,14 +11607,14 @@
     </row>
     <row r="38" spans="1:17" ht="14.1" customHeight="1">
       <c r="A38" s="33"/>
-      <c r="B38" s="385" t="s">
+      <c r="B38" s="434" t="s">
         <v>27</v>
       </c>
-      <c r="C38" s="385"/>
-      <c r="D38" s="385"/>
-      <c r="E38" s="385"/>
-      <c r="F38" s="385"/>
-      <c r="G38" s="385"/>
+      <c r="C38" s="434"/>
+      <c r="D38" s="434"/>
+      <c r="E38" s="434"/>
+      <c r="F38" s="434"/>
+      <c r="G38" s="434"/>
       <c r="H38" s="62"/>
       <c r="I38" s="45"/>
       <c r="J38" s="45"/>
@@ -11210,12 +11625,12 @@
     </row>
     <row r="39" spans="1:17" ht="14.1" customHeight="1">
       <c r="A39" s="57"/>
-      <c r="B39" s="386"/>
-      <c r="C39" s="386"/>
-      <c r="D39" s="386"/>
-      <c r="E39" s="386"/>
-      <c r="F39" s="386"/>
-      <c r="G39" s="386"/>
+      <c r="B39" s="435"/>
+      <c r="C39" s="435"/>
+      <c r="D39" s="435"/>
+      <c r="E39" s="435"/>
+      <c r="F39" s="435"/>
+      <c r="G39" s="435"/>
       <c r="H39" s="64"/>
       <c r="I39" s="64"/>
       <c r="J39" s="64"/>
@@ -11309,11 +11724,11 @@
       <c r="E46" s="180"/>
       <c r="F46" s="180"/>
       <c r="G46" s="181"/>
-      <c r="H46" s="380" t="s">
+      <c r="H46" s="429" t="s">
         <v>187</v>
       </c>
-      <c r="I46" s="380"/>
-      <c r="J46" s="380"/>
+      <c r="I46" s="429"/>
+      <c r="J46" s="429"/>
       <c r="K46" s="9"/>
     </row>
     <row r="47" spans="1:17" ht="14.1" customHeight="1" thickBot="1">
@@ -11332,17 +11747,6 @@
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="22">
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="H3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="G9:K9"/>
-    <mergeCell ref="B6:F8"/>
-    <mergeCell ref="G10:K12"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="H15:K16"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="B10:F12"/>
-    <mergeCell ref="B14:F17"/>
     <mergeCell ref="H46:J46"/>
     <mergeCell ref="H18:K18"/>
     <mergeCell ref="D19:F19"/>
@@ -11354,377 +11758,23 @@
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="B28:G28"/>
     <mergeCell ref="B30:G31"/>
+    <mergeCell ref="G10:K12"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="H15:K16"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="B10:F12"/>
+    <mergeCell ref="B14:F17"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="H3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="G9:K9"/>
+    <mergeCell ref="B6:F8"/>
   </mergeCells>
   <phoneticPr fontId="34" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.49" right="0.53" top="0.41" bottom="0.57999999999999996" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="72" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr>
-    <tabColor rgb="FFFFC000"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A5:P26"/>
-  <sheetFormatPr defaultColWidth="8.76953125" defaultRowHeight="14.25"/>
-  <cols>
-    <col min="1" max="1" width="8.76953125" style="73"/>
-    <col min="2" max="2" width="16.72265625" style="73" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.2265625" style="73" customWidth="1"/>
-    <col min="4" max="4" width="20.11328125" style="73" customWidth="1"/>
-    <col min="5" max="5" width="11.34375" style="73" customWidth="1"/>
-    <col min="6" max="6" width="8.06640625" style="73" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.41796875" style="73" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.703125" style="73" customWidth="1"/>
-    <col min="9" max="10" width="8.06640625" style="78" customWidth="1"/>
-    <col min="11" max="11" width="9.23828125" style="73" customWidth="1"/>
-    <col min="12" max="12" width="11.92578125" style="73" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.796875" style="73" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.875" style="73" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.00390625" style="73" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.86328125" style="73" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.76953125" style="73"/>
-  </cols>
-  <sheetData>
-    <row r="5" spans="1:16">
-      <c r="B5" s="74" t="str">
-        <f>'Commercial Invoice'!G5</f>
-        <v>INVOICE NO. :</v>
-      </c>
-      <c r="C5" s="74" t="str">
-        <f>'Commercial Invoice'!H5</f>
-        <v>OM4-DE-IS-0010</v>
-      </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="75"/>
-      <c r="F5" s="74"/>
-      <c r="G5" s="74"/>
-      <c r="H5" s="74"/>
-      <c r="I5" s="442"/>
-      <c r="J5" s="443"/>
-      <c r="K5" s="76" t="s">
-        <v>127</v>
-      </c>
-      <c r="L5" s="76"/>
-      <c r="M5" s="191">
-        <f>'Commercial Invoice'!H6</f>
-        <v>46177</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16">
-      <c r="B6" s="77"/>
-      <c r="C6" s="77"/>
-      <c r="D6" s="77"/>
-    </row>
-    <row r="7" spans="1:16" ht="47.25" customHeight="1">
-      <c r="A7" s="436" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="444" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="438" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="444" t="s">
-        <v>152</v>
-      </c>
-      <c r="E7" s="436" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7" s="440" t="s">
-        <v>153</v>
-      </c>
-      <c r="G7" s="441"/>
-      <c r="H7" s="436" t="s">
-        <v>154</v>
-      </c>
-      <c r="I7" s="436" t="s">
-        <v>161</v>
-      </c>
-      <c r="J7" s="436" t="s">
-        <v>160</v>
-      </c>
-      <c r="K7" s="436" t="s">
-        <v>155</v>
-      </c>
-      <c r="L7" s="436" t="s">
-        <v>156</v>
-      </c>
-      <c r="M7" s="438" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" ht="14.45" customHeight="1">
-      <c r="A8" s="437"/>
-      <c r="B8" s="445"/>
-      <c r="C8" s="439"/>
-      <c r="D8" s="445"/>
-      <c r="E8" s="437"/>
-      <c r="F8" s="200" t="s">
-        <v>158</v>
-      </c>
-      <c r="G8" s="200" t="s">
-        <v>159</v>
-      </c>
-      <c r="H8" s="437"/>
-      <c r="I8" s="437"/>
-      <c r="J8" s="437"/>
-      <c r="K8" s="437"/>
-      <c r="L8" s="437"/>
-      <c r="M8" s="439"/>
-      <c r="O8" s="73" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" ht="14.45" customHeight="1">
-      <c r="A9" s="262">
-        <v>1</v>
-      </c>
-      <c r="B9" s="290" t="s">
-        <v>201</v>
-      </c>
-      <c r="C9" s="349" t="s">
-        <v>205</v>
-      </c>
-      <c r="D9" s="268" t="s">
-        <v>163</v>
-      </c>
-      <c r="E9" s="290" t="s">
-        <v>198</v>
-      </c>
-      <c r="F9" s="350">
-        <f>'Detailed PL'!I15</f>
-        <v>32</v>
-      </c>
-      <c r="G9" s="351" t="str">
-        <f>'Detailed PL'!J15</f>
-        <v>EA</v>
-      </c>
-      <c r="H9" s="351" t="str">
-        <f>'Detailed PL'!K16</f>
-        <v>Wooden</v>
-      </c>
-      <c r="I9" s="352">
-        <f>'Detailed PL'!P16</f>
-        <v>576</v>
-      </c>
-      <c r="J9" s="352">
-        <f>'Detailed PL'!Q16</f>
-        <v>726</v>
-      </c>
-      <c r="K9" s="270">
-        <v>90.67</v>
-      </c>
-      <c r="L9" s="270">
-        <v>2901.44</v>
-      </c>
-      <c r="M9" s="270" t="s">
-        <v>197</v>
-      </c>
-      <c r="O9" s="342" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="14.45" customHeight="1">
-      <c r="A10" s="262">
-        <v>2</v>
-      </c>
-      <c r="B10" s="290" t="s">
-        <v>206</v>
-      </c>
-      <c r="C10" s="349" t="s">
-        <v>205</v>
-      </c>
-      <c r="D10" s="268" t="s">
-        <v>163</v>
-      </c>
-      <c r="E10" s="290" t="s">
-        <v>198</v>
-      </c>
-      <c r="F10" s="350">
-        <f>'Detailed PL'!I17</f>
-        <v>18</v>
-      </c>
-      <c r="G10" s="351" t="str">
-        <f>'Detailed PL'!J17</f>
-        <v>EA</v>
-      </c>
-      <c r="H10" s="351" t="str">
-        <f>'Detailed PL'!K18</f>
-        <v>Wooden</v>
-      </c>
-      <c r="I10" s="352">
-        <f>'Detailed PL'!P18</f>
-        <v>324</v>
-      </c>
-      <c r="J10" s="352">
-        <f>'Detailed PL'!Q18</f>
-        <v>474</v>
-      </c>
-      <c r="K10" s="270">
-        <v>90.68</v>
-      </c>
-      <c r="L10" s="270">
-        <v>1632.23</v>
-      </c>
-      <c r="M10" s="270" t="s">
-        <v>197</v>
-      </c>
-      <c r="O10" s="342" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="14.1" customHeight="1">
-      <c r="A11" s="82"/>
-      <c r="B11" s="83"/>
-      <c r="C11" s="84"/>
-      <c r="D11" s="84"/>
-      <c r="E11" s="85"/>
-      <c r="F11" s="86"/>
-      <c r="G11" s="86"/>
-      <c r="H11" s="87" t="s">
-        <v>32</v>
-      </c>
-      <c r="I11" s="88"/>
-      <c r="J11" s="84"/>
-      <c r="K11" s="84"/>
-      <c r="L11" s="327">
-        <f>SUM(L9:L10)</f>
-        <v>4533.67</v>
-      </c>
-      <c r="M11" s="89"/>
-      <c r="O11" s="343"/>
-      <c r="P11" s="342"/>
-    </row>
-    <row r="12" spans="1:16" ht="14.1" customHeight="1">
-      <c r="A12" s="90"/>
-      <c r="B12" s="91"/>
-      <c r="C12" s="81"/>
-      <c r="D12" s="81"/>
-      <c r="E12" s="92"/>
-      <c r="F12" s="93"/>
-      <c r="G12" s="93"/>
-      <c r="H12" s="93"/>
-      <c r="I12" s="94"/>
-      <c r="J12" s="94"/>
-      <c r="K12" s="81"/>
-      <c r="L12" s="81"/>
-      <c r="M12" s="91"/>
-      <c r="N12" s="80"/>
-      <c r="O12" s="80">
-        <f>L9+N19</f>
-        <v>5802.88</v>
-      </c>
-      <c r="P12" s="346"/>
-    </row>
-    <row r="13" spans="1:16">
-      <c r="O13" s="80">
-        <f>L10+N20</f>
-        <v>3264.4700000000003</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16">
-      <c r="N14" s="346"/>
-      <c r="O14" s="346"/>
-      <c r="P14" s="80"/>
-    </row>
-    <row r="15" spans="1:16">
-      <c r="N15" s="346"/>
-      <c r="O15" s="346"/>
-      <c r="P15" s="80"/>
-    </row>
-    <row r="16" spans="1:16">
-      <c r="L16" s="353">
-        <f>K9*F9</f>
-        <v>2901.44</v>
-      </c>
-      <c r="N16" s="346">
-        <f>F9*K9</f>
-        <v>2901.44</v>
-      </c>
-    </row>
-    <row r="17" spans="11:16">
-      <c r="L17" s="353">
-        <f>K10*F10</f>
-        <v>1632.2400000000002</v>
-      </c>
-      <c r="N17" s="346">
-        <f>F10*K10</f>
-        <v>1632.2400000000002</v>
-      </c>
-    </row>
-    <row r="18" spans="11:16">
-      <c r="K18" s="342"/>
-      <c r="L18" s="353">
-        <f>SUM(L16:L17)</f>
-        <v>4533.68</v>
-      </c>
-      <c r="N18" s="80"/>
-    </row>
-    <row r="19" spans="11:16">
-      <c r="K19" s="342"/>
-      <c r="L19" s="78"/>
-      <c r="N19" s="80">
-        <f>ROUND(N16,2)</f>
-        <v>2901.44</v>
-      </c>
-    </row>
-    <row r="20" spans="11:16">
-      <c r="K20" s="342"/>
-      <c r="L20" s="73">
-        <v>2901.55</v>
-      </c>
-      <c r="N20" s="80">
-        <f>ROUND(N17,2)</f>
-        <v>1632.24</v>
-      </c>
-      <c r="P20" s="356"/>
-    </row>
-    <row r="21" spans="11:16">
-      <c r="K21" s="342"/>
-      <c r="L21" s="73">
-        <v>1632.12</v>
-      </c>
-    </row>
-    <row r="22" spans="11:16">
-      <c r="L22" s="73">
-        <v>4533.67</v>
-      </c>
-    </row>
-    <row r="25" spans="11:16">
-      <c r="M25" s="346"/>
-    </row>
-    <row r="26" spans="11:16">
-      <c r="N26" s="367"/>
-      <c r="O26" s="367"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A8:N11" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <mergeCells count="13">
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="J7:J8"/>
-  </mergeCells>
-  <phoneticPr fontId="34" type="noConversion"/>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.70866141732283472" right="0.31496062992125984" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="67" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -11784,33 +11834,33 @@
     </row>
     <row r="3" spans="1:21" ht="37.5" customHeight="1">
       <c r="A3" s="10"/>
-      <c r="B3" s="422" t="s">
+      <c r="B3" s="390" t="s">
         <v>125</v>
       </c>
-      <c r="C3" s="459"/>
-      <c r="D3" s="459"/>
-      <c r="E3" s="459"/>
-      <c r="F3" s="459"/>
+      <c r="C3" s="456"/>
+      <c r="D3" s="456"/>
+      <c r="E3" s="456"/>
+      <c r="F3" s="456"/>
       <c r="G3" s="195"/>
-      <c r="H3" s="460"/>
-      <c r="I3" s="461"/>
-      <c r="J3" s="461"/>
-      <c r="K3" s="462"/>
+      <c r="H3" s="457"/>
+      <c r="I3" s="458"/>
+      <c r="J3" s="458"/>
+      <c r="K3" s="459"/>
     </row>
     <row r="4" spans="1:21" s="13" customFormat="1" ht="22.15" customHeight="1">
-      <c r="A4" s="425" t="s">
+      <c r="A4" s="393" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="426"/>
-      <c r="C4" s="426"/>
-      <c r="D4" s="426"/>
-      <c r="E4" s="426"/>
-      <c r="F4" s="426"/>
-      <c r="G4" s="426"/>
-      <c r="H4" s="426"/>
-      <c r="I4" s="426"/>
-      <c r="J4" s="426"/>
-      <c r="K4" s="427"/>
+      <c r="B4" s="394"/>
+      <c r="C4" s="394"/>
+      <c r="D4" s="394"/>
+      <c r="E4" s="394"/>
+      <c r="F4" s="394"/>
+      <c r="G4" s="394"/>
+      <c r="H4" s="394"/>
+      <c r="I4" s="394"/>
+      <c r="J4" s="394"/>
+      <c r="K4" s="395"/>
       <c r="L4" s="11"/>
       <c r="M4" s="11"/>
       <c r="N4" s="97"/>
@@ -11852,13 +11902,13 @@
     </row>
     <row r="6" spans="1:21" s="13" customFormat="1" ht="12.75">
       <c r="A6" s="99"/>
-      <c r="B6" s="454" t="s">
+      <c r="B6" s="481" t="s">
         <v>130</v>
       </c>
-      <c r="C6" s="455"/>
-      <c r="D6" s="455"/>
-      <c r="E6" s="455"/>
-      <c r="F6" s="456"/>
+      <c r="C6" s="482"/>
+      <c r="D6" s="482"/>
+      <c r="E6" s="482"/>
+      <c r="F6" s="483"/>
       <c r="G6" s="24" t="s">
         <v>4</v>
       </c>
@@ -11882,11 +11932,11 @@
     </row>
     <row r="7" spans="1:21" ht="12.75">
       <c r="A7" s="8"/>
-      <c r="B7" s="455"/>
-      <c r="C7" s="455"/>
-      <c r="D7" s="455"/>
-      <c r="E7" s="455"/>
-      <c r="F7" s="456"/>
+      <c r="B7" s="482"/>
+      <c r="C7" s="482"/>
+      <c r="D7" s="482"/>
+      <c r="E7" s="482"/>
+      <c r="F7" s="483"/>
       <c r="G7" s="29" t="s">
         <v>5</v>
       </c>
@@ -11899,11 +11949,11 @@
     </row>
     <row r="8" spans="1:21" ht="12.75">
       <c r="A8" s="8"/>
-      <c r="B8" s="457"/>
-      <c r="C8" s="457"/>
-      <c r="D8" s="457"/>
-      <c r="E8" s="457"/>
-      <c r="F8" s="458"/>
+      <c r="B8" s="484"/>
+      <c r="C8" s="484"/>
+      <c r="D8" s="484"/>
+      <c r="E8" s="484"/>
+      <c r="F8" s="485"/>
       <c r="G8" s="24" t="s">
         <v>4</v>
       </c>
@@ -11924,57 +11974,57 @@
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
       <c r="F9" s="34"/>
-      <c r="G9" s="428" t="str">
+      <c r="G9" s="396" t="str">
         <f>[6]CI!G9</f>
         <v>SHIPPING MARK</v>
       </c>
-      <c r="H9" s="429"/>
-      <c r="I9" s="429"/>
-      <c r="J9" s="429"/>
-      <c r="K9" s="430"/>
+      <c r="H9" s="397"/>
+      <c r="I9" s="397"/>
+      <c r="J9" s="397"/>
+      <c r="K9" s="398"/>
     </row>
     <row r="10" spans="1:21" ht="17.649999999999999" customHeight="1">
       <c r="A10" s="8"/>
-      <c r="B10" s="449" t="s">
+      <c r="B10" s="476" t="s">
         <v>128</v>
       </c>
-      <c r="C10" s="450"/>
-      <c r="D10" s="450"/>
-      <c r="E10" s="450"/>
-      <c r="F10" s="451"/>
-      <c r="G10" s="399" t="s">
+      <c r="C10" s="477"/>
+      <c r="D10" s="477"/>
+      <c r="E10" s="477"/>
+      <c r="F10" s="478"/>
+      <c r="G10" s="404" t="s">
         <v>9</v>
       </c>
-      <c r="H10" s="400"/>
-      <c r="I10" s="400"/>
-      <c r="J10" s="400"/>
-      <c r="K10" s="401"/>
+      <c r="H10" s="405"/>
+      <c r="I10" s="405"/>
+      <c r="J10" s="405"/>
+      <c r="K10" s="406"/>
     </row>
     <row r="11" spans="1:21" ht="17.649999999999999" customHeight="1">
       <c r="A11" s="8"/>
-      <c r="B11" s="450"/>
-      <c r="C11" s="450"/>
-      <c r="D11" s="450"/>
-      <c r="E11" s="450"/>
-      <c r="F11" s="451"/>
-      <c r="G11" s="402"/>
-      <c r="H11" s="403"/>
-      <c r="I11" s="403"/>
-      <c r="J11" s="403"/>
-      <c r="K11" s="404"/>
+      <c r="B11" s="477"/>
+      <c r="C11" s="477"/>
+      <c r="D11" s="477"/>
+      <c r="E11" s="477"/>
+      <c r="F11" s="478"/>
+      <c r="G11" s="407"/>
+      <c r="H11" s="408"/>
+      <c r="I11" s="408"/>
+      <c r="J11" s="408"/>
+      <c r="K11" s="409"/>
     </row>
     <row r="12" spans="1:21" ht="24" customHeight="1" thickBot="1">
       <c r="A12" s="35"/>
-      <c r="B12" s="452"/>
-      <c r="C12" s="452"/>
-      <c r="D12" s="452"/>
-      <c r="E12" s="452"/>
-      <c r="F12" s="453"/>
-      <c r="G12" s="405"/>
-      <c r="H12" s="406"/>
-      <c r="I12" s="406"/>
-      <c r="J12" s="406"/>
-      <c r="K12" s="407"/>
+      <c r="B12" s="479"/>
+      <c r="C12" s="479"/>
+      <c r="D12" s="479"/>
+      <c r="E12" s="479"/>
+      <c r="F12" s="480"/>
+      <c r="G12" s="410"/>
+      <c r="H12" s="411"/>
+      <c r="I12" s="411"/>
+      <c r="J12" s="411"/>
+      <c r="K12" s="412"/>
     </row>
     <row r="13" spans="1:21" ht="21.6" customHeight="1">
       <c r="A13" s="36" t="s">
@@ -11986,51 +12036,51 @@
       <c r="E13" s="180"/>
       <c r="F13" s="180"/>
       <c r="G13" s="101"/>
-      <c r="H13" s="473"/>
-      <c r="I13" s="473"/>
-      <c r="J13" s="473"/>
-      <c r="K13" s="474"/>
+      <c r="H13" s="470"/>
+      <c r="I13" s="470"/>
+      <c r="J13" s="470"/>
+      <c r="K13" s="471"/>
     </row>
     <row r="14" spans="1:21" ht="14.1" customHeight="1">
       <c r="A14" s="8"/>
-      <c r="B14" s="417" t="s">
+      <c r="B14" s="424" t="s">
         <v>131</v>
       </c>
-      <c r="C14" s="418"/>
-      <c r="D14" s="418"/>
-      <c r="E14" s="418"/>
-      <c r="F14" s="419"/>
+      <c r="C14" s="425"/>
+      <c r="D14" s="425"/>
+      <c r="E14" s="425"/>
+      <c r="F14" s="426"/>
       <c r="G14" s="38"/>
-      <c r="H14" s="408"/>
-      <c r="I14" s="408"/>
-      <c r="J14" s="408"/>
-      <c r="K14" s="409"/>
+      <c r="H14" s="413"/>
+      <c r="I14" s="413"/>
+      <c r="J14" s="413"/>
+      <c r="K14" s="414"/>
     </row>
     <row r="15" spans="1:21" ht="14.1" customHeight="1">
       <c r="A15" s="8"/>
-      <c r="B15" s="418"/>
-      <c r="C15" s="418"/>
-      <c r="D15" s="418"/>
-      <c r="E15" s="418"/>
-      <c r="F15" s="419"/>
+      <c r="B15" s="425"/>
+      <c r="C15" s="425"/>
+      <c r="D15" s="425"/>
+      <c r="E15" s="425"/>
+      <c r="F15" s="426"/>
       <c r="G15" s="274" t="s">
         <v>150</v>
       </c>
-      <c r="H15" s="410" t="str">
+      <c r="H15" s="415" t="str">
         <f>H5</f>
         <v>OM4-DE-IS-0010</v>
       </c>
-      <c r="I15" s="410"/>
-      <c r="J15" s="410"/>
+      <c r="I15" s="415"/>
+      <c r="J15" s="415"/>
       <c r="K15" s="275"/>
     </row>
     <row r="16" spans="1:21" ht="13.9" customHeight="1">
       <c r="A16" s="8"/>
-      <c r="B16" s="418"/>
-      <c r="C16" s="418"/>
-      <c r="D16" s="418"/>
-      <c r="E16" s="418"/>
-      <c r="F16" s="419"/>
+      <c r="B16" s="425"/>
+      <c r="C16" s="425"/>
+      <c r="D16" s="425"/>
+      <c r="E16" s="425"/>
+      <c r="F16" s="426"/>
       <c r="G16" s="38"/>
       <c r="H16" s="187"/>
       <c r="I16" s="187"/>
@@ -12039,19 +12089,19 @@
     </row>
     <row r="17" spans="1:22" ht="99.4" customHeight="1">
       <c r="A17" s="8"/>
-      <c r="B17" s="420"/>
-      <c r="C17" s="420"/>
-      <c r="D17" s="420"/>
-      <c r="E17" s="420"/>
-      <c r="F17" s="421"/>
+      <c r="B17" s="427"/>
+      <c r="C17" s="427"/>
+      <c r="D17" s="427"/>
+      <c r="E17" s="427"/>
+      <c r="F17" s="428"/>
       <c r="G17" s="274" t="s">
         <v>12</v>
       </c>
-      <c r="H17" s="475" t="s">
+      <c r="H17" s="472" t="s">
         <v>196</v>
       </c>
-      <c r="I17" s="475"/>
-      <c r="J17" s="475"/>
+      <c r="I17" s="472"/>
+      <c r="J17" s="472"/>
       <c r="K17" s="310"/>
     </row>
     <row r="18" spans="1:22" ht="18.600000000000001" customHeight="1">
@@ -12066,10 +12116,10 @@
       <c r="E18" s="30"/>
       <c r="F18" s="34"/>
       <c r="G18" s="38"/>
-      <c r="H18" s="465"/>
-      <c r="I18" s="465"/>
-      <c r="J18" s="465"/>
-      <c r="K18" s="466"/>
+      <c r="H18" s="462"/>
+      <c r="I18" s="462"/>
+      <c r="J18" s="462"/>
+      <c r="K18" s="463"/>
     </row>
     <row r="19" spans="1:22" s="6" customFormat="1" ht="12.75">
       <c r="A19" s="35"/>
@@ -12077,20 +12127,20 @@
         <v>210</v>
       </c>
       <c r="C19" s="261"/>
-      <c r="D19" s="383">
+      <c r="D19" s="432">
         <v>46208</v>
       </c>
-      <c r="E19" s="383"/>
-      <c r="F19" s="384"/>
+      <c r="E19" s="432"/>
+      <c r="F19" s="433"/>
       <c r="G19" s="174" t="s">
         <v>110</v>
       </c>
-      <c r="H19" s="467" t="s">
+      <c r="H19" s="464" t="s">
         <v>111</v>
       </c>
-      <c r="I19" s="467"/>
-      <c r="J19" s="467"/>
-      <c r="K19" s="468"/>
+      <c r="I19" s="464"/>
+      <c r="J19" s="464"/>
+      <c r="K19" s="465"/>
       <c r="M19" s="95"/>
       <c r="N19" s="66"/>
       <c r="O19" s="96"/>
@@ -12114,10 +12164,10 @@
       <c r="E20" s="30"/>
       <c r="F20" s="34"/>
       <c r="G20" s="37"/>
-      <c r="H20" s="465"/>
-      <c r="I20" s="465"/>
-      <c r="J20" s="465"/>
-      <c r="K20" s="466"/>
+      <c r="H20" s="462"/>
+      <c r="I20" s="462"/>
+      <c r="J20" s="462"/>
+      <c r="K20" s="463"/>
       <c r="M20" s="95"/>
       <c r="N20" s="66"/>
       <c r="O20" s="96"/>
@@ -12187,9 +12237,9 @@
       <c r="A23" s="35"/>
       <c r="B23" s="260"/>
       <c r="C23" s="261"/>
-      <c r="D23" s="389"/>
-      <c r="E23" s="389"/>
-      <c r="F23" s="390"/>
+      <c r="D23" s="436"/>
+      <c r="E23" s="436"/>
+      <c r="F23" s="437"/>
       <c r="G23" s="37"/>
       <c r="H23" s="181"/>
       <c r="I23" s="181"/>
@@ -12258,13 +12308,13 @@
     </row>
     <row r="26" spans="1:22" s="6" customFormat="1" ht="12.75">
       <c r="A26" s="35"/>
-      <c r="B26" s="391" t="s">
+      <c r="B26" s="438" t="s">
         <v>132</v>
       </c>
-      <c r="C26" s="391"/>
-      <c r="D26" s="391"/>
-      <c r="E26" s="391"/>
-      <c r="F26" s="392"/>
+      <c r="C26" s="438"/>
+      <c r="D26" s="438"/>
+      <c r="E26" s="438"/>
+      <c r="F26" s="439"/>
       <c r="G26" s="47"/>
       <c r="H26" s="48"/>
       <c r="I26" s="48"/>
@@ -12282,14 +12332,14 @@
       <c r="V26" s="7"/>
     </row>
     <row r="27" spans="1:22" s="28" customFormat="1" ht="35.25">
-      <c r="A27" s="469" t="s">
+      <c r="A27" s="466" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="470"/>
-      <c r="C27" s="470"/>
-      <c r="D27" s="470"/>
-      <c r="E27" s="470"/>
-      <c r="F27" s="470"/>
+      <c r="B27" s="467"/>
+      <c r="C27" s="467"/>
+      <c r="D27" s="467"/>
+      <c r="E27" s="467"/>
+      <c r="F27" s="467"/>
       <c r="G27" s="102" t="s">
         <v>21</v>
       </c>
@@ -12314,13 +12364,13 @@
     </row>
     <row r="28" spans="1:22" ht="52.9" customHeight="1">
       <c r="A28" s="36"/>
-      <c r="B28" s="471" t="s">
+      <c r="B28" s="468" t="s">
         <v>134</v>
       </c>
-      <c r="C28" s="471"/>
-      <c r="D28" s="471"/>
-      <c r="E28" s="471"/>
-      <c r="F28" s="472"/>
+      <c r="C28" s="468"/>
+      <c r="D28" s="468"/>
+      <c r="E28" s="468"/>
+      <c r="F28" s="469"/>
       <c r="G28" s="53"/>
       <c r="H28" s="53"/>
       <c r="I28" s="109"/>
@@ -12341,14 +12391,14 @@
       <c r="K29" s="285"/>
     </row>
     <row r="30" spans="1:22" ht="14.1" customHeight="1">
-      <c r="A30" s="446" t="s">
+      <c r="A30" s="473" t="s">
         <v>200</v>
       </c>
-      <c r="B30" s="447"/>
-      <c r="C30" s="447"/>
-      <c r="D30" s="447"/>
-      <c r="E30" s="447"/>
-      <c r="F30" s="448"/>
+      <c r="B30" s="474"/>
+      <c r="C30" s="474"/>
+      <c r="D30" s="474"/>
+      <c r="E30" s="474"/>
+      <c r="F30" s="475"/>
       <c r="G30" s="357"/>
       <c r="H30" s="357"/>
       <c r="I30" s="284"/>
@@ -12356,12 +12406,12 @@
       <c r="K30" s="285"/>
     </row>
     <row r="31" spans="1:22" ht="14.1" customHeight="1">
-      <c r="A31" s="447"/>
-      <c r="B31" s="447"/>
-      <c r="C31" s="447"/>
-      <c r="D31" s="447"/>
-      <c r="E31" s="447"/>
-      <c r="F31" s="448"/>
+      <c r="A31" s="474"/>
+      <c r="B31" s="474"/>
+      <c r="C31" s="474"/>
+      <c r="D31" s="474"/>
+      <c r="E31" s="474"/>
+      <c r="F31" s="475"/>
       <c r="G31" s="284" t="s">
         <v>146</v>
       </c>
@@ -12383,12 +12433,12 @@
       </c>
     </row>
     <row r="32" spans="1:22" ht="14.1" customHeight="1">
-      <c r="A32" s="447"/>
-      <c r="B32" s="447"/>
-      <c r="C32" s="447"/>
-      <c r="D32" s="447"/>
-      <c r="E32" s="447"/>
-      <c r="F32" s="448"/>
+      <c r="A32" s="474"/>
+      <c r="B32" s="474"/>
+      <c r="C32" s="474"/>
+      <c r="D32" s="474"/>
+      <c r="E32" s="474"/>
+      <c r="F32" s="475"/>
       <c r="G32" s="284" t="s">
         <v>146</v>
       </c>
@@ -12493,10 +12543,10 @@
       <c r="D38" s="112"/>
       <c r="E38" s="112"/>
       <c r="F38" s="112"/>
-      <c r="G38" s="463" t="s">
+      <c r="G38" s="460" t="s">
         <v>38</v>
       </c>
-      <c r="H38" s="464"/>
+      <c r="H38" s="461"/>
       <c r="I38" s="359">
         <f>SUM(I28:I37)</f>
         <v>900</v>
@@ -12714,11 +12764,11 @@
       <c r="E47" s="180"/>
       <c r="F47" s="180"/>
       <c r="G47" s="188"/>
-      <c r="H47" s="380" t="s">
+      <c r="H47" s="429" t="s">
         <v>187</v>
       </c>
-      <c r="I47" s="380"/>
-      <c r="J47" s="380"/>
+      <c r="I47" s="429"/>
+      <c r="J47" s="429"/>
       <c r="K47" s="9"/>
       <c r="M47" s="95"/>
       <c r="N47" s="66"/>
@@ -12756,6 +12806,14 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="H47:J47"/>
+    <mergeCell ref="A30:F32"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="G9:K9"/>
+    <mergeCell ref="G10:K12"/>
+    <mergeCell ref="B10:F12"/>
+    <mergeCell ref="B6:F8"/>
+    <mergeCell ref="H15:J15"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="H3:K3"/>
     <mergeCell ref="G38:H38"/>
@@ -12771,14 +12829,6 @@
     <mergeCell ref="B14:F17"/>
     <mergeCell ref="H13:K13"/>
     <mergeCell ref="H17:J17"/>
-    <mergeCell ref="H47:J47"/>
-    <mergeCell ref="A30:F32"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="G9:K9"/>
-    <mergeCell ref="G10:K12"/>
-    <mergeCell ref="B10:F12"/>
-    <mergeCell ref="B6:F8"/>
-    <mergeCell ref="H15:J15"/>
   </mergeCells>
   <phoneticPr fontId="34" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -12860,15 +12910,15 @@
     </row>
     <row r="3" spans="2:20" ht="27.6" customHeight="1" thickBot="1">
       <c r="B3" s="199"/>
-      <c r="C3" s="480" t="s">
+      <c r="C3" s="492" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="480"/>
-      <c r="E3" s="480"/>
-      <c r="F3" s="480"/>
-      <c r="G3" s="480"/>
-      <c r="H3" s="480"/>
-      <c r="I3" s="480"/>
+      <c r="D3" s="492"/>
+      <c r="E3" s="492"/>
+      <c r="F3" s="492"/>
+      <c r="G3" s="492"/>
+      <c r="H3" s="492"/>
+      <c r="I3" s="492"/>
       <c r="J3" s="181"/>
       <c r="K3" s="182"/>
       <c r="L3" s="117"/>
@@ -12882,27 +12932,27 @@
       <c r="T3" s="199"/>
     </row>
     <row r="4" spans="2:20" ht="33.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="B4" s="481" t="s">
+      <c r="B4" s="493" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="482"/>
-      <c r="D4" s="482"/>
-      <c r="E4" s="482"/>
-      <c r="F4" s="482"/>
-      <c r="G4" s="482"/>
-      <c r="H4" s="482"/>
-      <c r="I4" s="482"/>
-      <c r="J4" s="482"/>
-      <c r="K4" s="482"/>
-      <c r="L4" s="482"/>
-      <c r="M4" s="482"/>
-      <c r="N4" s="482"/>
-      <c r="O4" s="482"/>
-      <c r="P4" s="482"/>
-      <c r="Q4" s="482"/>
-      <c r="R4" s="482"/>
-      <c r="S4" s="482"/>
-      <c r="T4" s="483"/>
+      <c r="C4" s="494"/>
+      <c r="D4" s="494"/>
+      <c r="E4" s="494"/>
+      <c r="F4" s="494"/>
+      <c r="G4" s="494"/>
+      <c r="H4" s="494"/>
+      <c r="I4" s="494"/>
+      <c r="J4" s="494"/>
+      <c r="K4" s="494"/>
+      <c r="L4" s="494"/>
+      <c r="M4" s="494"/>
+      <c r="N4" s="494"/>
+      <c r="O4" s="494"/>
+      <c r="P4" s="494"/>
+      <c r="Q4" s="494"/>
+      <c r="R4" s="494"/>
+      <c r="S4" s="494"/>
+      <c r="T4" s="495"/>
     </row>
     <row r="5" spans="2:20" s="7" customFormat="1" ht="17.25" customHeight="1" thickTop="1">
       <c r="B5" s="66"/>
@@ -13144,68 +13194,68 @@
       <c r="T12" s="66"/>
     </row>
     <row r="13" spans="2:20" s="28" customFormat="1" ht="20.25" customHeight="1">
-      <c r="B13" s="476" t="s">
+      <c r="B13" s="488" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="484" t="s">
+      <c r="C13" s="496" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="486" t="s">
+      <c r="D13" s="498" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="476" t="s">
+      <c r="E13" s="488" t="s">
         <v>145</v>
       </c>
-      <c r="F13" s="478" t="s">
+      <c r="F13" s="490" t="s">
         <v>72</v>
       </c>
-      <c r="G13" s="479"/>
-      <c r="H13" s="476" t="s">
+      <c r="G13" s="491"/>
+      <c r="H13" s="488" t="s">
         <v>73</v>
       </c>
-      <c r="I13" s="478" t="s">
+      <c r="I13" s="490" t="s">
         <v>74</v>
       </c>
-      <c r="J13" s="470"/>
-      <c r="K13" s="470"/>
-      <c r="L13" s="479"/>
-      <c r="M13" s="476" t="s">
+      <c r="J13" s="467"/>
+      <c r="K13" s="467"/>
+      <c r="L13" s="491"/>
+      <c r="M13" s="488" t="s">
         <v>75</v>
       </c>
-      <c r="N13" s="476" t="s">
+      <c r="N13" s="488" t="s">
         <v>76</v>
       </c>
-      <c r="O13" s="476" t="s">
+      <c r="O13" s="488" t="s">
         <v>77</v>
       </c>
-      <c r="P13" s="488" t="s">
+      <c r="P13" s="486" t="s">
         <v>140</v>
       </c>
-      <c r="Q13" s="488" t="s">
+      <c r="Q13" s="486" t="s">
         <v>141</v>
       </c>
-      <c r="R13" s="488" t="s">
+      <c r="R13" s="486" t="s">
         <v>142</v>
       </c>
-      <c r="S13" s="476" t="s">
+      <c r="S13" s="488" t="s">
         <v>78</v>
       </c>
-      <c r="T13" s="476" t="s">
+      <c r="T13" s="488" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="14" spans="2:20" s="28" customFormat="1" ht="33" customHeight="1">
-      <c r="B14" s="477"/>
-      <c r="C14" s="485"/>
-      <c r="D14" s="487"/>
-      <c r="E14" s="477"/>
+      <c r="B14" s="489"/>
+      <c r="C14" s="497"/>
+      <c r="D14" s="499"/>
+      <c r="E14" s="489"/>
       <c r="F14" s="126" t="s">
         <v>80</v>
       </c>
       <c r="G14" s="126" t="s">
         <v>81</v>
       </c>
-      <c r="H14" s="477"/>
+      <c r="H14" s="489"/>
       <c r="I14" s="127" t="s">
         <v>82</v>
       </c>
@@ -13218,14 +13268,14 @@
       <c r="L14" s="127" t="s">
         <v>85</v>
       </c>
-      <c r="M14" s="477"/>
-      <c r="N14" s="477"/>
-      <c r="O14" s="477"/>
-      <c r="P14" s="489"/>
-      <c r="Q14" s="489"/>
-      <c r="R14" s="489"/>
-      <c r="S14" s="477"/>
-      <c r="T14" s="477"/>
+      <c r="M14" s="489"/>
+      <c r="N14" s="489"/>
+      <c r="O14" s="489"/>
+      <c r="P14" s="487"/>
+      <c r="Q14" s="487"/>
+      <c r="R14" s="487"/>
+      <c r="S14" s="489"/>
+      <c r="T14" s="489"/>
     </row>
     <row r="15" spans="2:20" s="7" customFormat="1" ht="47.25" customHeight="1">
       <c r="B15" s="208" t="s">
@@ -13364,18 +13414,18 @@
       </c>
     </row>
     <row r="17" spans="2:20" ht="18.75" customHeight="1">
-      <c r="B17" s="478" t="s">
+      <c r="B17" s="490" t="s">
         <v>86</v>
       </c>
-      <c r="C17" s="470"/>
-      <c r="D17" s="470"/>
-      <c r="E17" s="470"/>
-      <c r="F17" s="470"/>
-      <c r="G17" s="470"/>
-      <c r="H17" s="470"/>
-      <c r="I17" s="470"/>
-      <c r="J17" s="470"/>
-      <c r="K17" s="479"/>
+      <c r="C17" s="467"/>
+      <c r="D17" s="467"/>
+      <c r="E17" s="467"/>
+      <c r="F17" s="467"/>
+      <c r="G17" s="467"/>
+      <c r="H17" s="467"/>
+      <c r="I17" s="467"/>
+      <c r="J17" s="467"/>
+      <c r="K17" s="491"/>
       <c r="L17" s="291">
         <f>SUM(L15:L16)</f>
         <v>3.1680000000000001</v>
@@ -13437,6 +13487,8 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="T13:T14"/>
+    <mergeCell ref="P13:P14"/>
     <mergeCell ref="Q13:Q14"/>
     <mergeCell ref="R13:R14"/>
     <mergeCell ref="S13:S14"/>
@@ -13453,8 +13505,6 @@
     <mergeCell ref="M13:M14"/>
     <mergeCell ref="N13:N14"/>
     <mergeCell ref="O13:O14"/>
-    <mergeCell ref="T13:T14"/>
-    <mergeCell ref="P13:P14"/>
   </mergeCells>
   <phoneticPr fontId="34" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -13493,47 +13543,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="91.15" customHeight="1" thickBot="1">
-      <c r="A1" s="515" t="s">
+      <c r="A1" s="506" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="515"/>
-      <c r="C1" s="515"/>
-      <c r="D1" s="515"/>
-      <c r="E1" s="515"/>
-      <c r="F1" s="515"/>
-      <c r="G1" s="515"/>
-      <c r="H1" s="515"/>
-      <c r="I1" s="515"/>
-      <c r="J1" s="515"/>
+      <c r="B1" s="506"/>
+      <c r="C1" s="506"/>
+      <c r="D1" s="506"/>
+      <c r="E1" s="506"/>
+      <c r="F1" s="506"/>
+      <c r="G1" s="506"/>
+      <c r="H1" s="506"/>
+      <c r="I1" s="506"/>
+      <c r="J1" s="506"/>
     </row>
     <row r="2" spans="1:13" ht="32.65" customHeight="1">
-      <c r="A2" s="516" t="s">
+      <c r="A2" s="507" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="517"/>
-      <c r="C2" s="517"/>
-      <c r="D2" s="517"/>
-      <c r="E2" s="517"/>
-      <c r="F2" s="517"/>
-      <c r="G2" s="517"/>
-      <c r="H2" s="517"/>
-      <c r="I2" s="517"/>
-      <c r="J2" s="518"/>
+      <c r="B2" s="508"/>
+      <c r="C2" s="508"/>
+      <c r="D2" s="508"/>
+      <c r="E2" s="508"/>
+      <c r="F2" s="508"/>
+      <c r="G2" s="508"/>
+      <c r="H2" s="508"/>
+      <c r="I2" s="508"/>
+      <c r="J2" s="509"/>
     </row>
     <row r="3" spans="1:13" ht="28.15" customHeight="1">
-      <c r="A3" s="519" t="str">
+      <c r="A3" s="510" t="str">
         <f>[6]CI!B26</f>
         <v>Address: O Mon Power Complex at Phuoc Thoi wards, O Mon district, Can Tho city</v>
       </c>
-      <c r="B3" s="520"/>
-      <c r="C3" s="520"/>
-      <c r="D3" s="520"/>
-      <c r="E3" s="520"/>
-      <c r="F3" s="520"/>
-      <c r="G3" s="520"/>
-      <c r="H3" s="520"/>
-      <c r="I3" s="520"/>
-      <c r="J3" s="521"/>
+      <c r="B3" s="511"/>
+      <c r="C3" s="511"/>
+      <c r="D3" s="511"/>
+      <c r="E3" s="511"/>
+      <c r="F3" s="511"/>
+      <c r="G3" s="511"/>
+      <c r="H3" s="511"/>
+      <c r="I3" s="511"/>
+      <c r="J3" s="512"/>
     </row>
     <row r="5" spans="1:13" s="162" customFormat="1" ht="40.15" customHeight="1">
       <c r="A5" s="176" t="s">
@@ -13542,16 +13592,16 @@
       <c r="B5" s="161" t="s">
         <v>97</v>
       </c>
-      <c r="C5" s="522" t="s">
+      <c r="C5" s="513" t="s">
         <v>135</v>
       </c>
-      <c r="D5" s="523"/>
-      <c r="E5" s="523"/>
-      <c r="F5" s="523"/>
-      <c r="G5" s="523"/>
-      <c r="H5" s="523"/>
-      <c r="I5" s="523"/>
-      <c r="J5" s="524"/>
+      <c r="D5" s="514"/>
+      <c r="E5" s="514"/>
+      <c r="F5" s="514"/>
+      <c r="G5" s="514"/>
+      <c r="H5" s="514"/>
+      <c r="I5" s="514"/>
+      <c r="J5" s="515"/>
     </row>
     <row r="6" spans="1:13" s="162" customFormat="1" ht="55.5" customHeight="1">
       <c r="A6" s="177" t="s">
@@ -13560,16 +13610,16 @@
       <c r="B6" s="163" t="s">
         <v>97</v>
       </c>
-      <c r="C6" s="513" t="s">
+      <c r="C6" s="504" t="s">
         <v>136</v>
       </c>
-      <c r="D6" s="513"/>
-      <c r="E6" s="513"/>
-      <c r="F6" s="513"/>
-      <c r="G6" s="513"/>
-      <c r="H6" s="513"/>
-      <c r="I6" s="513"/>
-      <c r="J6" s="514"/>
+      <c r="D6" s="504"/>
+      <c r="E6" s="504"/>
+      <c r="F6" s="504"/>
+      <c r="G6" s="504"/>
+      <c r="H6" s="504"/>
+      <c r="I6" s="504"/>
+      <c r="J6" s="505"/>
     </row>
     <row r="7" spans="1:13" s="162" customFormat="1" ht="94.15" customHeight="1">
       <c r="A7" s="177" t="s">
@@ -13578,16 +13628,16 @@
       <c r="B7" s="164" t="s">
         <v>97</v>
       </c>
-      <c r="C7" s="513" t="s">
+      <c r="C7" s="504" t="s">
         <v>137</v>
       </c>
-      <c r="D7" s="513"/>
-      <c r="E7" s="513"/>
-      <c r="F7" s="513"/>
-      <c r="G7" s="513"/>
-      <c r="H7" s="513"/>
-      <c r="I7" s="513"/>
-      <c r="J7" s="514"/>
+      <c r="D7" s="504"/>
+      <c r="E7" s="504"/>
+      <c r="F7" s="504"/>
+      <c r="G7" s="504"/>
+      <c r="H7" s="504"/>
+      <c r="I7" s="504"/>
+      <c r="J7" s="505"/>
     </row>
     <row r="8" spans="1:13" s="162" customFormat="1" ht="20.65" customHeight="1">
       <c r="A8" s="177" t="s">
@@ -13596,52 +13646,52 @@
       <c r="B8" s="164" t="s">
         <v>100</v>
       </c>
-      <c r="C8" s="513" t="s">
+      <c r="C8" s="504" t="s">
         <v>138</v>
       </c>
-      <c r="D8" s="513"/>
-      <c r="E8" s="513"/>
-      <c r="F8" s="513"/>
-      <c r="G8" s="513"/>
-      <c r="H8" s="513"/>
-      <c r="I8" s="513"/>
-      <c r="J8" s="514"/>
+      <c r="D8" s="504"/>
+      <c r="E8" s="504"/>
+      <c r="F8" s="504"/>
+      <c r="G8" s="504"/>
+      <c r="H8" s="504"/>
+      <c r="I8" s="504"/>
+      <c r="J8" s="505"/>
     </row>
     <row r="9" spans="1:13" s="162" customFormat="1" ht="20.65" customHeight="1">
       <c r="A9" s="177"/>
       <c r="B9" s="164"/>
-      <c r="C9" s="513"/>
-      <c r="D9" s="513"/>
-      <c r="E9" s="513"/>
-      <c r="F9" s="513"/>
-      <c r="G9" s="513"/>
-      <c r="H9" s="513"/>
-      <c r="I9" s="513"/>
-      <c r="J9" s="514"/>
+      <c r="C9" s="504"/>
+      <c r="D9" s="504"/>
+      <c r="E9" s="504"/>
+      <c r="F9" s="504"/>
+      <c r="G9" s="504"/>
+      <c r="H9" s="504"/>
+      <c r="I9" s="504"/>
+      <c r="J9" s="505"/>
     </row>
     <row r="10" spans="1:13" s="162" customFormat="1" ht="20.65" customHeight="1">
       <c r="A10" s="177"/>
       <c r="B10" s="164"/>
-      <c r="C10" s="513"/>
-      <c r="D10" s="513"/>
-      <c r="E10" s="513"/>
-      <c r="F10" s="513"/>
-      <c r="G10" s="513"/>
-      <c r="H10" s="513"/>
-      <c r="I10" s="513"/>
-      <c r="J10" s="514"/>
+      <c r="C10" s="504"/>
+      <c r="D10" s="504"/>
+      <c r="E10" s="504"/>
+      <c r="F10" s="504"/>
+      <c r="G10" s="504"/>
+      <c r="H10" s="504"/>
+      <c r="I10" s="504"/>
+      <c r="J10" s="505"/>
     </row>
     <row r="11" spans="1:13" s="162" customFormat="1" ht="171" customHeight="1">
       <c r="A11" s="177"/>
       <c r="B11" s="164"/>
-      <c r="C11" s="513"/>
-      <c r="D11" s="513"/>
-      <c r="E11" s="513"/>
-      <c r="F11" s="513"/>
-      <c r="G11" s="513"/>
-      <c r="H11" s="513"/>
-      <c r="I11" s="513"/>
-      <c r="J11" s="514"/>
+      <c r="C11" s="504"/>
+      <c r="D11" s="504"/>
+      <c r="E11" s="504"/>
+      <c r="F11" s="504"/>
+      <c r="G11" s="504"/>
+      <c r="H11" s="504"/>
+      <c r="I11" s="504"/>
+      <c r="J11" s="505"/>
     </row>
     <row r="12" spans="1:13" s="162" customFormat="1">
       <c r="A12" s="177" t="s">
@@ -13650,16 +13700,16 @@
       <c r="B12" s="163" t="s">
         <v>97</v>
       </c>
-      <c r="C12" s="513" t="s">
+      <c r="C12" s="504" t="s">
         <v>115</v>
       </c>
-      <c r="D12" s="513"/>
-      <c r="E12" s="513"/>
-      <c r="F12" s="513"/>
-      <c r="G12" s="513"/>
-      <c r="H12" s="513"/>
-      <c r="I12" s="513"/>
-      <c r="J12" s="514"/>
+      <c r="D12" s="504"/>
+      <c r="E12" s="504"/>
+      <c r="F12" s="504"/>
+      <c r="G12" s="504"/>
+      <c r="H12" s="504"/>
+      <c r="I12" s="504"/>
+      <c r="J12" s="505"/>
     </row>
     <row r="13" spans="1:13" s="303" customFormat="1" ht="25.5">
       <c r="A13" s="266" t="s">
@@ -13668,11 +13718,11 @@
       <c r="B13" s="267" t="s">
         <v>100</v>
       </c>
-      <c r="C13" s="525" t="s">
+      <c r="C13" s="516" t="s">
         <v>199</v>
       </c>
-      <c r="D13" s="525"/>
-      <c r="E13" s="525"/>
+      <c r="D13" s="516"/>
+      <c r="E13" s="516"/>
       <c r="F13" s="300"/>
       <c r="G13" s="301"/>
       <c r="H13" s="301"/>
@@ -13686,17 +13736,17 @@
       <c r="B14" s="163" t="s">
         <v>97</v>
       </c>
-      <c r="C14" s="511" t="str">
+      <c r="C14" s="502" t="str">
         <f>[6]CI!B28</f>
         <v>PLANT/ EQUIPMENT AND MATERIALS FOR O MON IV THERMAL</v>
       </c>
-      <c r="D14" s="511"/>
-      <c r="E14" s="511"/>
-      <c r="F14" s="511"/>
-      <c r="G14" s="511"/>
-      <c r="H14" s="511"/>
-      <c r="I14" s="511"/>
-      <c r="J14" s="512"/>
+      <c r="D14" s="502"/>
+      <c r="E14" s="502"/>
+      <c r="F14" s="502"/>
+      <c r="G14" s="502"/>
+      <c r="H14" s="502"/>
+      <c r="I14" s="502"/>
+      <c r="J14" s="503"/>
     </row>
     <row r="15" spans="1:13" s="162" customFormat="1">
       <c r="A15" s="266" t="s">
@@ -13705,17 +13755,17 @@
       <c r="B15" s="267" t="s">
         <v>97</v>
       </c>
-      <c r="C15" s="509" t="str">
+      <c r="C15" s="500" t="str">
         <f>'PL(2_2)'!D15</f>
         <v>Zinc Primer Paint</v>
       </c>
-      <c r="D15" s="509"/>
-      <c r="E15" s="509"/>
-      <c r="F15" s="509"/>
-      <c r="G15" s="509"/>
-      <c r="H15" s="509"/>
-      <c r="I15" s="509"/>
-      <c r="J15" s="510"/>
+      <c r="D15" s="500"/>
+      <c r="E15" s="500"/>
+      <c r="F15" s="500"/>
+      <c r="G15" s="500"/>
+      <c r="H15" s="500"/>
+      <c r="I15" s="500"/>
+      <c r="J15" s="501"/>
       <c r="L15" s="162" t="s">
         <v>186</v>
       </c>
@@ -14142,47 +14192,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="91.15" customHeight="1" thickBot="1">
-      <c r="A1" s="515" t="s">
+      <c r="A1" s="506" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="515"/>
-      <c r="C1" s="515"/>
-      <c r="D1" s="515"/>
-      <c r="E1" s="515"/>
-      <c r="F1" s="515"/>
-      <c r="G1" s="515"/>
-      <c r="H1" s="515"/>
-      <c r="I1" s="515"/>
-      <c r="J1" s="515"/>
+      <c r="B1" s="506"/>
+      <c r="C1" s="506"/>
+      <c r="D1" s="506"/>
+      <c r="E1" s="506"/>
+      <c r="F1" s="506"/>
+      <c r="G1" s="506"/>
+      <c r="H1" s="506"/>
+      <c r="I1" s="506"/>
+      <c r="J1" s="506"/>
     </row>
     <row r="2" spans="1:13" ht="32.65" customHeight="1">
-      <c r="A2" s="516" t="s">
+      <c r="A2" s="507" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="517"/>
-      <c r="C2" s="517"/>
-      <c r="D2" s="517"/>
-      <c r="E2" s="517"/>
-      <c r="F2" s="517"/>
-      <c r="G2" s="517"/>
-      <c r="H2" s="517"/>
-      <c r="I2" s="517"/>
-      <c r="J2" s="518"/>
+      <c r="B2" s="508"/>
+      <c r="C2" s="508"/>
+      <c r="D2" s="508"/>
+      <c r="E2" s="508"/>
+      <c r="F2" s="508"/>
+      <c r="G2" s="508"/>
+      <c r="H2" s="508"/>
+      <c r="I2" s="508"/>
+      <c r="J2" s="509"/>
     </row>
     <row r="3" spans="1:13" ht="28.15" customHeight="1">
-      <c r="A3" s="519" t="str">
+      <c r="A3" s="510" t="str">
         <f>[6]CI!B26</f>
         <v>Address: O Mon Power Complex at Phuoc Thoi wards, O Mon district, Can Tho city</v>
       </c>
-      <c r="B3" s="520"/>
-      <c r="C3" s="520"/>
-      <c r="D3" s="520"/>
-      <c r="E3" s="520"/>
-      <c r="F3" s="520"/>
-      <c r="G3" s="520"/>
-      <c r="H3" s="520"/>
-      <c r="I3" s="520"/>
-      <c r="J3" s="521"/>
+      <c r="B3" s="511"/>
+      <c r="C3" s="511"/>
+      <c r="D3" s="511"/>
+      <c r="E3" s="511"/>
+      <c r="F3" s="511"/>
+      <c r="G3" s="511"/>
+      <c r="H3" s="511"/>
+      <c r="I3" s="511"/>
+      <c r="J3" s="512"/>
     </row>
     <row r="5" spans="1:13" s="162" customFormat="1" ht="40.15" customHeight="1">
       <c r="A5" s="176" t="s">
@@ -14191,16 +14241,16 @@
       <c r="B5" s="161" t="s">
         <v>97</v>
       </c>
-      <c r="C5" s="522" t="s">
+      <c r="C5" s="513" t="s">
         <v>135</v>
       </c>
-      <c r="D5" s="523"/>
-      <c r="E5" s="523"/>
-      <c r="F5" s="523"/>
-      <c r="G5" s="523"/>
-      <c r="H5" s="523"/>
-      <c r="I5" s="523"/>
-      <c r="J5" s="524"/>
+      <c r="D5" s="514"/>
+      <c r="E5" s="514"/>
+      <c r="F5" s="514"/>
+      <c r="G5" s="514"/>
+      <c r="H5" s="514"/>
+      <c r="I5" s="514"/>
+      <c r="J5" s="515"/>
     </row>
     <row r="6" spans="1:13" s="162" customFormat="1" ht="55.5" customHeight="1">
       <c r="A6" s="177" t="s">
@@ -14209,16 +14259,16 @@
       <c r="B6" s="163" t="s">
         <v>97</v>
       </c>
-      <c r="C6" s="513" t="s">
+      <c r="C6" s="504" t="s">
         <v>136</v>
       </c>
-      <c r="D6" s="513"/>
-      <c r="E6" s="513"/>
-      <c r="F6" s="513"/>
-      <c r="G6" s="513"/>
-      <c r="H6" s="513"/>
-      <c r="I6" s="513"/>
-      <c r="J6" s="514"/>
+      <c r="D6" s="504"/>
+      <c r="E6" s="504"/>
+      <c r="F6" s="504"/>
+      <c r="G6" s="504"/>
+      <c r="H6" s="504"/>
+      <c r="I6" s="504"/>
+      <c r="J6" s="505"/>
     </row>
     <row r="7" spans="1:13" s="162" customFormat="1" ht="94.15" customHeight="1">
       <c r="A7" s="177" t="s">
@@ -14227,16 +14277,16 @@
       <c r="B7" s="164" t="s">
         <v>97</v>
       </c>
-      <c r="C7" s="513" t="s">
+      <c r="C7" s="504" t="s">
         <v>137</v>
       </c>
-      <c r="D7" s="513"/>
-      <c r="E7" s="513"/>
-      <c r="F7" s="513"/>
-      <c r="G7" s="513"/>
-      <c r="H7" s="513"/>
-      <c r="I7" s="513"/>
-      <c r="J7" s="514"/>
+      <c r="D7" s="504"/>
+      <c r="E7" s="504"/>
+      <c r="F7" s="504"/>
+      <c r="G7" s="504"/>
+      <c r="H7" s="504"/>
+      <c r="I7" s="504"/>
+      <c r="J7" s="505"/>
     </row>
     <row r="8" spans="1:13" s="162" customFormat="1" ht="20.65" customHeight="1">
       <c r="A8" s="177" t="s">
@@ -14245,52 +14295,52 @@
       <c r="B8" s="164" t="s">
         <v>100</v>
       </c>
-      <c r="C8" s="513" t="s">
+      <c r="C8" s="504" t="s">
         <v>138</v>
       </c>
-      <c r="D8" s="513"/>
-      <c r="E8" s="513"/>
-      <c r="F8" s="513"/>
-      <c r="G8" s="513"/>
-      <c r="H8" s="513"/>
-      <c r="I8" s="513"/>
-      <c r="J8" s="514"/>
+      <c r="D8" s="504"/>
+      <c r="E8" s="504"/>
+      <c r="F8" s="504"/>
+      <c r="G8" s="504"/>
+      <c r="H8" s="504"/>
+      <c r="I8" s="504"/>
+      <c r="J8" s="505"/>
     </row>
     <row r="9" spans="1:13" s="162" customFormat="1" ht="20.65" customHeight="1">
       <c r="A9" s="177"/>
       <c r="B9" s="164"/>
-      <c r="C9" s="513"/>
-      <c r="D9" s="513"/>
-      <c r="E9" s="513"/>
-      <c r="F9" s="513"/>
-      <c r="G9" s="513"/>
-      <c r="H9" s="513"/>
-      <c r="I9" s="513"/>
-      <c r="J9" s="514"/>
+      <c r="C9" s="504"/>
+      <c r="D9" s="504"/>
+      <c r="E9" s="504"/>
+      <c r="F9" s="504"/>
+      <c r="G9" s="504"/>
+      <c r="H9" s="504"/>
+      <c r="I9" s="504"/>
+      <c r="J9" s="505"/>
     </row>
     <row r="10" spans="1:13" s="162" customFormat="1" ht="20.65" customHeight="1">
       <c r="A10" s="177"/>
       <c r="B10" s="164"/>
-      <c r="C10" s="513"/>
-      <c r="D10" s="513"/>
-      <c r="E10" s="513"/>
-      <c r="F10" s="513"/>
-      <c r="G10" s="513"/>
-      <c r="H10" s="513"/>
-      <c r="I10" s="513"/>
-      <c r="J10" s="514"/>
+      <c r="C10" s="504"/>
+      <c r="D10" s="504"/>
+      <c r="E10" s="504"/>
+      <c r="F10" s="504"/>
+      <c r="G10" s="504"/>
+      <c r="H10" s="504"/>
+      <c r="I10" s="504"/>
+      <c r="J10" s="505"/>
     </row>
     <row r="11" spans="1:13" s="162" customFormat="1" ht="171" customHeight="1">
       <c r="A11" s="177"/>
       <c r="B11" s="164"/>
-      <c r="C11" s="513"/>
-      <c r="D11" s="513"/>
-      <c r="E11" s="513"/>
-      <c r="F11" s="513"/>
-      <c r="G11" s="513"/>
-      <c r="H11" s="513"/>
-      <c r="I11" s="513"/>
-      <c r="J11" s="514"/>
+      <c r="C11" s="504"/>
+      <c r="D11" s="504"/>
+      <c r="E11" s="504"/>
+      <c r="F11" s="504"/>
+      <c r="G11" s="504"/>
+      <c r="H11" s="504"/>
+      <c r="I11" s="504"/>
+      <c r="J11" s="505"/>
     </row>
     <row r="12" spans="1:13" s="162" customFormat="1">
       <c r="A12" s="177" t="s">
@@ -14299,16 +14349,16 @@
       <c r="B12" s="163" t="s">
         <v>97</v>
       </c>
-      <c r="C12" s="513" t="s">
+      <c r="C12" s="504" t="s">
         <v>115</v>
       </c>
-      <c r="D12" s="513"/>
-      <c r="E12" s="513"/>
-      <c r="F12" s="513"/>
-      <c r="G12" s="513"/>
-      <c r="H12" s="513"/>
-      <c r="I12" s="513"/>
-      <c r="J12" s="514"/>
+      <c r="D12" s="504"/>
+      <c r="E12" s="504"/>
+      <c r="F12" s="504"/>
+      <c r="G12" s="504"/>
+      <c r="H12" s="504"/>
+      <c r="I12" s="504"/>
+      <c r="J12" s="505"/>
     </row>
     <row r="13" spans="1:13" s="303" customFormat="1" ht="25.5">
       <c r="A13" s="266" t="s">
@@ -14317,11 +14367,11 @@
       <c r="B13" s="267" t="s">
         <v>100</v>
       </c>
-      <c r="C13" s="525" t="s">
+      <c r="C13" s="516" t="s">
         <v>199</v>
       </c>
-      <c r="D13" s="525"/>
-      <c r="E13" s="525"/>
+      <c r="D13" s="516"/>
+      <c r="E13" s="516"/>
       <c r="F13" s="300"/>
       <c r="G13" s="301"/>
       <c r="H13" s="301"/>
@@ -14335,17 +14385,17 @@
       <c r="B14" s="163" t="s">
         <v>97</v>
       </c>
-      <c r="C14" s="511" t="str">
+      <c r="C14" s="502" t="str">
         <f>[6]CI!B28</f>
         <v>PLANT/ EQUIPMENT AND MATERIALS FOR O MON IV THERMAL</v>
       </c>
-      <c r="D14" s="511"/>
-      <c r="E14" s="511"/>
-      <c r="F14" s="511"/>
-      <c r="G14" s="511"/>
-      <c r="H14" s="511"/>
-      <c r="I14" s="511"/>
-      <c r="J14" s="512"/>
+      <c r="D14" s="502"/>
+      <c r="E14" s="502"/>
+      <c r="F14" s="502"/>
+      <c r="G14" s="502"/>
+      <c r="H14" s="502"/>
+      <c r="I14" s="502"/>
+      <c r="J14" s="503"/>
     </row>
     <row r="15" spans="1:13" s="162" customFormat="1">
       <c r="A15" s="266" t="s">
@@ -14354,17 +14404,17 @@
       <c r="B15" s="267" t="s">
         <v>97</v>
       </c>
-      <c r="C15" s="509" t="str">
+      <c r="C15" s="500" t="str">
         <f>'PL(2_2)'!D16</f>
         <v>Zinc Primer Paint, Sealant</v>
       </c>
-      <c r="D15" s="509"/>
-      <c r="E15" s="509"/>
-      <c r="F15" s="509"/>
-      <c r="G15" s="509"/>
-      <c r="H15" s="509"/>
-      <c r="I15" s="509"/>
-      <c r="J15" s="510"/>
+      <c r="D15" s="500"/>
+      <c r="E15" s="500"/>
+      <c r="F15" s="500"/>
+      <c r="G15" s="500"/>
+      <c r="H15" s="500"/>
+      <c r="I15" s="500"/>
+      <c r="J15" s="501"/>
       <c r="L15" s="162" t="s">
         <v>186</v>
       </c>
@@ -14746,17 +14796,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="C8:J11"/>
+    <mergeCell ref="C12:J12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C14:J14"/>
+    <mergeCell ref="C15:J15"/>
     <mergeCell ref="C7:J7"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="C5:J5"/>
     <mergeCell ref="C6:J6"/>
-    <mergeCell ref="C8:J11"/>
-    <mergeCell ref="C12:J12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C14:J14"/>
-    <mergeCell ref="C15:J15"/>
   </mergeCells>
   <phoneticPr fontId="34" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -14830,16 +14880,16 @@
       <c r="J5" s="218"/>
     </row>
     <row r="6" spans="1:10" ht="35.25" customHeight="1">
-      <c r="A6" s="369" t="s">
+      <c r="A6" s="376" t="s">
         <v>173</v>
       </c>
-      <c r="B6" s="369"/>
-      <c r="C6" s="369"/>
-      <c r="D6" s="369"/>
-      <c r="E6" s="369"/>
-      <c r="F6" s="369"/>
-      <c r="G6" s="369"/>
-      <c r="H6" s="369"/>
+      <c r="B6" s="376"/>
+      <c r="C6" s="376"/>
+      <c r="D6" s="376"/>
+      <c r="E6" s="376"/>
+      <c r="F6" s="376"/>
+      <c r="G6" s="376"/>
+      <c r="H6" s="376"/>
     </row>
     <row r="7" spans="1:10" s="136" customFormat="1" ht="20.25" customHeight="1" thickBot="1">
       <c r="A7" s="223" t="s">
@@ -14858,33 +14908,33 @@
       <c r="J7" s="224"/>
     </row>
     <row r="8" spans="1:10" s="227" customFormat="1" ht="21.95" customHeight="1">
-      <c r="A8" s="370" t="s">
+      <c r="A8" s="518" t="s">
         <v>175</v>
       </c>
-      <c r="B8" s="372" t="s">
+      <c r="B8" s="520" t="s">
         <v>176</v>
       </c>
-      <c r="C8" s="372" t="s">
+      <c r="C8" s="520" t="s">
         <v>177</v>
       </c>
-      <c r="D8" s="374" t="s">
+      <c r="D8" s="522" t="s">
         <v>178</v>
       </c>
-      <c r="E8" s="375"/>
-      <c r="F8" s="376" t="s">
+      <c r="E8" s="523"/>
+      <c r="F8" s="524" t="s">
         <v>179</v>
       </c>
-      <c r="G8" s="377"/>
-      <c r="H8" s="378" t="s">
+      <c r="G8" s="525"/>
+      <c r="H8" s="526" t="s">
         <v>180</v>
       </c>
       <c r="I8" s="226"/>
       <c r="J8" s="226"/>
     </row>
     <row r="9" spans="1:10" s="227" customFormat="1" ht="21.95" customHeight="1">
-      <c r="A9" s="371"/>
-      <c r="B9" s="373"/>
-      <c r="C9" s="373"/>
+      <c r="A9" s="519"/>
+      <c r="B9" s="521"/>
+      <c r="C9" s="521"/>
       <c r="D9" s="317" t="s">
         <v>181</v>
       </c>
@@ -14897,7 +14947,7 @@
       <c r="G9" s="228" t="s">
         <v>184</v>
       </c>
-      <c r="H9" s="379"/>
+      <c r="H9" s="527"/>
       <c r="I9" s="226"/>
       <c r="J9" s="226"/>
     </row>
@@ -15281,8 +15331,8 @@
       <c r="J44" s="218"/>
     </row>
     <row r="45" spans="1:18" s="217" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B45" s="368"/>
-      <c r="C45" s="368"/>
+      <c r="B45" s="517"/>
+      <c r="C45" s="517"/>
       <c r="D45" s="246"/>
       <c r="E45" s="220"/>
       <c r="F45" s="247"/>

</xml_diff>